<commit_message>
Atualiza dados da homologacao - 10/07/2026 14:30
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dataprevrj-my.sharepoint.com/personal/thiago_delima_dataprev_gov_br/Documents/Área de Trabalho/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="8_{AE89E8CF-B2D9-4866-89EB-E71F2B0AB318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D5E19C4D-8438-4D45-92A2-D55A548376FB}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C00F6A8-AFD7-44F3-8533-95644DBA44F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cenários homologação" sheetId="6" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="216">
   <si>
     <t>PENDENTE</t>
   </si>
@@ -181,12 +181,6 @@
     <t>Atividade fora do conjunto {1..5} descaracteriza</t>
   </si>
   <si>
-    <t>X</t>
-  </si>
-  <si>
-    <t>CANCELADO - O próprio banco de dados impede esse tipo de situação</t>
-  </si>
-  <si>
     <t>CT-031</t>
   </si>
   <si>
@@ -293,10 +287,6 @@
   </si>
   <si>
     <t>Requerente não encontrado no grupo familiar</t>
-  </si>
-  <si>
-    <t>Verificar CAF dos outros membros da família informados na AD
-Avaliar pra próxima versão</t>
   </si>
   <si>
     <t>CT-060</t>
@@ -511,12 +501,6 @@
     <t>Menor completa 16 durante o período - descaracterização parcial</t>
   </si>
   <si>
-    <t>Levar em consideração a mão-de-obra "não"</t>
-  </si>
-  <si>
-    <t>CANCELADO - O próprio CAF considera mão-de-obra como "não" para menor de idade</t>
-  </si>
-  <si>
     <t>CT-089</t>
   </si>
   <si>
@@ -536,10 +520,6 @@
   </si>
   <si>
     <t>Dependência de serviço externo (Receita) - pode ser testado com mock</t>
-  </si>
-  <si>
-    <t>Considerar que se a mão-de-obra for "sim", a pessoa com certeza será maior de 16 anos
-Daí não precisa avaliar a idade</t>
   </si>
   <si>
     <t>CT-093</t>
@@ -1100,21 +1080,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C39B64EC-B305-411B-89CD-90AE48303B1A}">
-  <dimension ref="A1:K44"/>
+  <dimension ref="A1:I44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="31.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.109375" customWidth="1"/>
     <col min="4" max="4" width="76.88671875" customWidth="1"/>
     <col min="5" max="5" width="22.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="20.88671875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="38.44140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="32.109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="89" customWidth="1"/>
-    <col min="10" max="10" width="56.109375" customWidth="1"/>
+    <col min="9" max="9" width="107.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>1</v>
       </c>
@@ -1143,7 +1122,13 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>204</v>
+      </c>
+      <c r="B2" t="s">
+        <v>201</v>
+      </c>
       <c r="C2" t="s">
         <v>10</v>
       </c>
@@ -1166,7 +1151,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C3" t="s">
         <v>16</v>
       </c>
@@ -1189,7 +1174,13 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>210</v>
+      </c>
+      <c r="B4" t="s">
+        <v>201</v>
+      </c>
       <c r="C4" t="s">
         <v>23</v>
       </c>
@@ -1212,7 +1203,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C5" t="s">
         <v>28</v>
       </c>
@@ -1235,7 +1226,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C6" t="s">
         <v>35</v>
       </c>
@@ -1258,7 +1249,10 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="B7" t="s">
+        <v>209</v>
+      </c>
       <c r="C7" t="s">
         <v>38</v>
       </c>
@@ -1280,212 +1274,200 @@
       <c r="I7" t="s">
         <v>43</v>
       </c>
-      <c r="J7" t="s">
+    </row>
+    <row r="8" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C8" t="s">
         <v>44</v>
       </c>
-      <c r="K7" t="s">
+      <c r="D8" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="C8" t="s">
+      <c r="E8" t="s">
         <v>46</v>
-      </c>
-      <c r="D8" t="s">
-        <v>47</v>
-      </c>
-      <c r="E8" t="s">
-        <v>48</v>
       </c>
       <c r="F8" t="s">
         <v>31</v>
       </c>
       <c r="G8" t="s">
+        <v>47</v>
+      </c>
+      <c r="H8" t="s">
+        <v>48</v>
+      </c>
+      <c r="I8" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="H8" t="s">
+    </row>
+    <row r="9" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C9" t="s">
         <v>50</v>
       </c>
-      <c r="I8" s="1" t="s">
+      <c r="D9" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="C9" t="s">
-        <v>52</v>
-      </c>
-      <c r="D9" t="s">
-        <v>53</v>
-      </c>
       <c r="E9" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F9" t="s">
         <v>0</v>
       </c>
       <c r="G9" t="s">
+        <v>52</v>
+      </c>
+      <c r="H9" t="s">
+        <v>48</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C10" t="s">
         <v>54</v>
       </c>
-      <c r="H9" t="s">
-        <v>50</v>
-      </c>
-      <c r="I9" s="1" t="s">
+      <c r="D10" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="C10" t="s">
+      <c r="E10" t="s">
         <v>56</v>
-      </c>
-      <c r="D10" t="s">
-        <v>57</v>
-      </c>
-      <c r="E10" t="s">
-        <v>58</v>
       </c>
       <c r="F10" t="s">
         <v>31</v>
       </c>
       <c r="G10" t="s">
+        <v>57</v>
+      </c>
+      <c r="H10" t="s">
+        <v>58</v>
+      </c>
+      <c r="I10" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="H10" t="s">
+    </row>
+    <row r="11" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C11" t="s">
         <v>60</v>
       </c>
-      <c r="I10" s="1" t="s">
+      <c r="D11" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="C11" t="s">
-        <v>62</v>
-      </c>
-      <c r="D11" t="s">
-        <v>63</v>
-      </c>
       <c r="E11" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F11" t="s">
         <v>31</v>
       </c>
       <c r="G11" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H11" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="I11" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="C12" t="s">
+        <v>63</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="C12" t="s">
+      <c r="E12" t="s">
+        <v>56</v>
+      </c>
+      <c r="F12" t="s">
         <v>65</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="G12" t="s">
         <v>66</v>
       </c>
-      <c r="E12" t="s">
+      <c r="H12" t="s">
         <v>58</v>
       </c>
-      <c r="F12" t="s">
+      <c r="I12" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="G12" t="s">
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="C13" t="s">
         <v>68</v>
       </c>
-      <c r="H12" t="s">
-        <v>60</v>
-      </c>
-      <c r="I12" s="1" t="s">
+      <c r="D13" t="s">
         <v>69</v>
       </c>
-      <c r="J12" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="C13" t="s">
+      <c r="E13" t="s">
         <v>70</v>
-      </c>
-      <c r="D13" t="s">
-        <v>71</v>
-      </c>
-      <c r="E13" t="s">
-        <v>72</v>
       </c>
       <c r="F13" t="s">
         <v>31</v>
       </c>
       <c r="G13" t="s">
+        <v>71</v>
+      </c>
+      <c r="H13" t="s">
+        <v>72</v>
+      </c>
+      <c r="I13" t="s">
         <v>73</v>
       </c>
-      <c r="H13" t="s">
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="C14" t="s">
         <v>74</v>
       </c>
-      <c r="I13" t="s">
+      <c r="D14" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="C14" t="s">
-        <v>76</v>
-      </c>
-      <c r="D14" t="s">
-        <v>77</v>
-      </c>
       <c r="E14" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F14" s="4" t="s">
         <v>19</v>
       </c>
       <c r="G14" t="s">
+        <v>76</v>
+      </c>
+      <c r="H14" t="s">
+        <v>72</v>
+      </c>
+      <c r="I14" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="C15" t="s">
         <v>78</v>
       </c>
-      <c r="H14" t="s">
-        <v>74</v>
-      </c>
-      <c r="I14" t="s">
+      <c r="D15" t="s">
         <v>79</v>
       </c>
-      <c r="J14" s="1" t="s">
+      <c r="E15" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="C15" t="s">
+      <c r="F15" t="s">
+        <v>65</v>
+      </c>
+      <c r="G15" t="s">
+        <v>66</v>
+      </c>
+      <c r="H15" t="s">
         <v>81</v>
       </c>
-      <c r="D15" t="s">
+      <c r="I15" t="s">
         <v>82</v>
       </c>
-      <c r="E15" t="s">
+    </row>
+    <row r="16" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C16" t="s">
         <v>83</v>
       </c>
-      <c r="F15" t="s">
-        <v>67</v>
-      </c>
-      <c r="G15" t="s">
-        <v>68</v>
-      </c>
-      <c r="H15" t="s">
+      <c r="D16" t="s">
         <v>84</v>
       </c>
-      <c r="I15" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="C16" t="s">
-        <v>86</v>
-      </c>
-      <c r="D16" t="s">
-        <v>87</v>
-      </c>
       <c r="E16" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F16" t="s">
         <v>31</v>
@@ -1494,21 +1476,21 @@
         <v>32</v>
       </c>
       <c r="H16" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="17" spans="3:11" x14ac:dyDescent="0.3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="17" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C17" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="D17" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="E17" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F17" t="s">
         <v>0</v>
@@ -1517,661 +1499,640 @@
         <v>25</v>
       </c>
       <c r="H17" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="I17" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="18" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C18" t="s">
+        <v>89</v>
+      </c>
+      <c r="D18" t="s">
+        <v>90</v>
+      </c>
+      <c r="E18" t="s">
+        <v>80</v>
+      </c>
+      <c r="F18" t="s">
+        <v>65</v>
+      </c>
+      <c r="G18" t="s">
+        <v>66</v>
+      </c>
+      <c r="H18" t="s">
+        <v>81</v>
+      </c>
+      <c r="I18" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="18" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="C18" t="s">
+    <row r="19" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C19" t="s">
         <v>92</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D19" t="s">
         <v>93</v>
       </c>
-      <c r="E18" t="s">
-        <v>83</v>
-      </c>
-      <c r="F18" t="s">
-        <v>67</v>
-      </c>
-      <c r="G18" t="s">
-        <v>68</v>
-      </c>
-      <c r="H18" t="s">
-        <v>84</v>
-      </c>
-      <c r="I18" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="19" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="C19" t="s">
-        <v>95</v>
-      </c>
-      <c r="D19" t="s">
-        <v>96</v>
-      </c>
       <c r="E19" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F19" t="s">
         <v>31</v>
       </c>
       <c r="G19" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H19" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="I19" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="20" spans="3:11" ht="28.8" x14ac:dyDescent="0.3">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="20" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C20" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="D20" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="E20" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F20" s="4" t="s">
         <v>19</v>
       </c>
       <c r="G20" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="H20" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="I20" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="21" spans="2:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C21" t="s">
+        <v>98</v>
+      </c>
+      <c r="D21" t="s">
+        <v>99</v>
+      </c>
+      <c r="E21" t="s">
         <v>100</v>
       </c>
-      <c r="J20" s="1" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="21" spans="3:11" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="C21" t="s">
+      <c r="F21" t="s">
         <v>101</v>
       </c>
-      <c r="D21" t="s">
+      <c r="G21" t="s">
         <v>102</v>
       </c>
-      <c r="E21" t="s">
+      <c r="H21" t="s">
         <v>103</v>
       </c>
-      <c r="F21" t="s">
+      <c r="I21" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="G21" t="s">
+    </row>
+    <row r="22" spans="2:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C22" t="s">
         <v>105</v>
       </c>
-      <c r="H21" t="s">
+      <c r="D22" t="s">
         <v>106</v>
       </c>
-      <c r="I21" s="1" t="s">
+      <c r="E22" t="s">
+        <v>100</v>
+      </c>
+      <c r="F22" t="s">
+        <v>65</v>
+      </c>
+      <c r="G22" t="s">
+        <v>66</v>
+      </c>
+      <c r="H22" t="s">
+        <v>103</v>
+      </c>
+      <c r="I22" s="1" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="22" spans="3:11" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="C22" t="s">
+    <row r="23" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C23" t="s">
         <v>108</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D23" t="s">
         <v>109</v>
       </c>
-      <c r="E22" t="s">
-        <v>103</v>
-      </c>
-      <c r="F22" t="s">
-        <v>67</v>
-      </c>
-      <c r="G22" t="s">
-        <v>68</v>
-      </c>
-      <c r="H22" t="s">
-        <v>106</v>
-      </c>
-      <c r="I22" s="1" t="s">
+      <c r="E23" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="23" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="C23" t="s">
+      <c r="F23" t="s">
+        <v>101</v>
+      </c>
+      <c r="G23" t="s">
         <v>111</v>
       </c>
-      <c r="D23" t="s">
+      <c r="H23" t="s">
         <v>112</v>
       </c>
-      <c r="E23" t="s">
+      <c r="I23" t="s">
         <v>113</v>
       </c>
-      <c r="F23" t="s">
-        <v>104</v>
-      </c>
-      <c r="G23" t="s">
+    </row>
+    <row r="24" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C24" t="s">
         <v>114</v>
       </c>
-      <c r="H23" t="s">
+      <c r="D24" t="s">
         <v>115</v>
       </c>
-      <c r="I23" t="s">
+      <c r="E24" t="s">
+        <v>110</v>
+      </c>
+      <c r="F24" t="s">
+        <v>65</v>
+      </c>
+      <c r="G24" t="s">
+        <v>66</v>
+      </c>
+      <c r="H24" t="s">
+        <v>112</v>
+      </c>
+      <c r="I24" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="24" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="C24" t="s">
+    <row r="25" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C25" t="s">
         <v>117</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D25" t="s">
         <v>118</v>
       </c>
-      <c r="E24" t="s">
-        <v>113</v>
-      </c>
-      <c r="F24" t="s">
-        <v>67</v>
-      </c>
-      <c r="G24" t="s">
-        <v>68</v>
-      </c>
-      <c r="H24" t="s">
-        <v>115</v>
-      </c>
-      <c r="I24" t="s">
+      <c r="E25" t="s">
         <v>119</v>
-      </c>
-    </row>
-    <row r="25" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="C25" t="s">
-        <v>120</v>
-      </c>
-      <c r="D25" t="s">
-        <v>121</v>
-      </c>
-      <c r="E25" t="s">
-        <v>122</v>
       </c>
       <c r="F25" t="s">
         <v>19</v>
       </c>
       <c r="G25" t="s">
+        <v>120</v>
+      </c>
+      <c r="H25" t="s">
+        <v>121</v>
+      </c>
+      <c r="I25" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="26" spans="2:9" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="C26" t="s">
         <v>123</v>
       </c>
-      <c r="H25" t="s">
+      <c r="D26" t="s">
         <v>124</v>
       </c>
-      <c r="I25" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="26" spans="3:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="C26" t="s">
-        <v>126</v>
-      </c>
-      <c r="D26" t="s">
-        <v>127</v>
-      </c>
       <c r="E26" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="F26" t="s">
         <v>31</v>
       </c>
       <c r="G26" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="H26" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="27" spans="3:11" x14ac:dyDescent="0.3">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="27" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C27" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="D27" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="E27" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="F27" t="s">
         <v>31</v>
       </c>
       <c r="G27" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="H27" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I27" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="28" spans="3:11" x14ac:dyDescent="0.3">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="28" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C28" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="D28" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="E28" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="F28" t="s">
         <v>31</v>
       </c>
       <c r="G28" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="H28" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I28" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="29" spans="3:11" x14ac:dyDescent="0.3">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="29" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C29" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="D29" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="E29" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="F29" t="s">
         <v>19</v>
       </c>
       <c r="G29" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="H29" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I29" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="30" spans="3:11" x14ac:dyDescent="0.3">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="30" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C30" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D30" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="E30" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="F30" t="s">
         <v>31</v>
       </c>
       <c r="G30" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="H30" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I30" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="31" spans="3:11" x14ac:dyDescent="0.3">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="31" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C31" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="D31" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="E31" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="F31" t="s">
         <v>31</v>
       </c>
       <c r="G31" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="H31" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I31" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="32" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B32" t="s">
+        <v>209</v>
+      </c>
+      <c r="C32" t="s">
+        <v>141</v>
+      </c>
+      <c r="D32" t="s">
+        <v>142</v>
+      </c>
+      <c r="E32" t="s">
         <v>143</v>
-      </c>
-    </row>
-    <row r="32" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="C32" t="s">
-        <v>144</v>
-      </c>
-      <c r="D32" t="s">
-        <v>145</v>
-      </c>
-      <c r="E32" t="s">
-        <v>146</v>
       </c>
       <c r="F32" t="s">
         <v>31</v>
       </c>
       <c r="G32" t="s">
+        <v>144</v>
+      </c>
+      <c r="H32" t="s">
+        <v>145</v>
+      </c>
+      <c r="I32" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="33" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B33" t="s">
+        <v>209</v>
+      </c>
+      <c r="C33" t="s">
         <v>147</v>
       </c>
-      <c r="H32" t="s">
+      <c r="D33" t="s">
         <v>148</v>
       </c>
-      <c r="I32" t="s">
-        <v>149</v>
-      </c>
-      <c r="J32" t="s">
-        <v>150</v>
-      </c>
-      <c r="K32" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="33" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="C33" t="s">
-        <v>152</v>
-      </c>
-      <c r="D33" t="s">
-        <v>153</v>
-      </c>
       <c r="E33" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="F33" t="s">
         <v>31</v>
       </c>
       <c r="G33" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="H33" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="I33" t="s">
-        <v>154</v>
-      </c>
-      <c r="J33" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="34" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B34" t="s">
+        <v>209</v>
+      </c>
+      <c r="C34" t="s">
         <v>150</v>
       </c>
-      <c r="K33" t="s">
+      <c r="D34" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="34" spans="3:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="C34" t="s">
-        <v>155</v>
-      </c>
-      <c r="D34" t="s">
-        <v>156</v>
-      </c>
       <c r="E34" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="F34" t="s">
         <v>0</v>
       </c>
       <c r="G34" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="H34" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="I34" t="s">
-        <v>158</v>
-      </c>
-      <c r="J34" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="K34" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="35" spans="3:11" x14ac:dyDescent="0.3">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="35" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C35" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="D35" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="E35" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="F35" t="s">
         <v>19</v>
       </c>
       <c r="G35" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="H35" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="I35" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="36" spans="3:11" x14ac:dyDescent="0.3">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="36" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C36" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="D36" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="E36" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="F36" t="s">
         <v>0</v>
       </c>
       <c r="G36" t="s">
+        <v>157</v>
+      </c>
+      <c r="H36" t="s">
+        <v>158</v>
+      </c>
+      <c r="I36" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="37" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C37" t="s">
         <v>163</v>
       </c>
-      <c r="H36" t="s">
+      <c r="D37" t="s">
         <v>164</v>
       </c>
-      <c r="I36" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="37" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="C37" t="s">
-        <v>169</v>
-      </c>
-      <c r="D37" t="s">
-        <v>170</v>
-      </c>
       <c r="E37" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="F37" t="s">
         <v>19</v>
       </c>
       <c r="G37" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="H37" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="I37" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="38" spans="3:11" ht="100.8" x14ac:dyDescent="0.3">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="38" spans="2:9" ht="100.8" x14ac:dyDescent="0.3">
       <c r="C38" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="E38" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="F38" t="s">
         <v>19</v>
       </c>
       <c r="G38" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="H38" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="I38" t="s">
-        <v>174</v>
-      </c>
-      <c r="J38" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="39" spans="3:11" x14ac:dyDescent="0.3">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="39" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C39" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="D39" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="E39" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="F39" t="s">
         <v>19</v>
       </c>
       <c r="G39" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="H39" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="I39" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="40" spans="3:11" x14ac:dyDescent="0.3">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="40" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C40" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="D40" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="E40" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="F40" t="s">
         <v>19</v>
       </c>
       <c r="G40" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="H40" t="s">
+        <v>172</v>
+      </c>
+      <c r="I40" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="41" spans="2:9" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="C41" t="s">
+        <v>177</v>
+      </c>
+      <c r="D41" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="I40" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="41" spans="3:11" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="C41" t="s">
-        <v>183</v>
-      </c>
-      <c r="D41" s="1" t="s">
-        <v>184</v>
-      </c>
       <c r="E41" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="F41" t="s">
         <v>19</v>
       </c>
       <c r="G41" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="H41" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="I41" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="42" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C42" t="s">
+        <v>180</v>
+      </c>
+      <c r="D42" t="s">
+        <v>181</v>
+      </c>
+      <c r="E42" t="s">
+        <v>182</v>
+      </c>
+      <c r="F42" t="s">
+        <v>101</v>
+      </c>
+      <c r="G42" t="s">
+        <v>183</v>
+      </c>
+      <c r="H42" t="s">
+        <v>184</v>
+      </c>
+      <c r="I42" t="s">
         <v>185</v>
       </c>
-      <c r="J41" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="42" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="C42" t="s">
+    </row>
+    <row r="43" spans="2:9" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="C43" t="s">
         <v>186</v>
       </c>
-      <c r="D42" t="s">
+      <c r="D43" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="E42" t="s">
+      <c r="E43" t="s">
+        <v>182</v>
+      </c>
+      <c r="F43" t="s">
+        <v>101</v>
+      </c>
+      <c r="G43" t="s">
         <v>188</v>
       </c>
-      <c r="F42" t="s">
-        <v>104</v>
-      </c>
-      <c r="G42" t="s">
+      <c r="H43" t="s">
+        <v>184</v>
+      </c>
+      <c r="I43" t="s">
         <v>189</v>
       </c>
-      <c r="H42" t="s">
+    </row>
+    <row r="44" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C44" t="s">
         <v>190</v>
       </c>
-      <c r="I42" t="s">
+      <c r="D44" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="43" spans="3:11" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="C43" t="s">
+      <c r="E44" t="s">
+        <v>182</v>
+      </c>
+      <c r="F44" t="s">
+        <v>65</v>
+      </c>
+      <c r="G44" t="s">
+        <v>66</v>
+      </c>
+      <c r="H44" t="s">
+        <v>184</v>
+      </c>
+      <c r="I44" t="s">
         <v>192</v>
-      </c>
-      <c r="D43" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="E43" t="s">
-        <v>188</v>
-      </c>
-      <c r="F43" t="s">
-        <v>104</v>
-      </c>
-      <c r="G43" t="s">
-        <v>194</v>
-      </c>
-      <c r="H43" t="s">
-        <v>190</v>
-      </c>
-      <c r="I43" t="s">
-        <v>195</v>
-      </c>
-      <c r="J43" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="44" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="C44" t="s">
-        <v>196</v>
-      </c>
-      <c r="D44" t="s">
-        <v>197</v>
-      </c>
-      <c r="E44" t="s">
-        <v>188</v>
-      </c>
-      <c r="F44" t="s">
-        <v>67</v>
-      </c>
-      <c r="G44" t="s">
-        <v>68</v>
-      </c>
-      <c r="H44" t="s">
-        <v>190</v>
-      </c>
-      <c r="I44" t="s">
-        <v>198</v>
       </c>
     </row>
   </sheetData>
@@ -2210,19 +2171,19 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="B1" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="C1" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="D1" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="E1" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="G1" t="s">
         <v>2</v>
@@ -2230,74 +2191,74 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="G2" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="G3" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="G4" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="C5" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="G5" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="C6" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="G6" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="C7" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="G7" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza dados da homologacao - 10/07/2026 14:45
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C00F6A8-AFD7-44F3-8533-95644DBA44F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD6959C8-4363-4CBC-B6AA-45BB84C12559}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cenários homologação" sheetId="6" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="216">
   <si>
     <t>PENDENTE</t>
   </si>
@@ -1152,6 +1152,12 @@
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>202</v>
+      </c>
+      <c r="B3" t="s">
+        <v>203</v>
+      </c>
       <c r="C3" t="s">
         <v>16</v>
       </c>
@@ -1250,6 +1256,9 @@
       </c>
     </row>
     <row r="7" spans="1:9" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>204</v>
+      </c>
       <c r="B7" t="s">
         <v>209</v>
       </c>
@@ -1482,7 +1491,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C17" t="s">
         <v>86</v>
       </c>
@@ -1505,7 +1514,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="18" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C18" t="s">
         <v>89</v>
       </c>
@@ -1528,7 +1537,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C19" t="s">
         <v>92</v>
       </c>
@@ -1551,7 +1560,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C20" t="s">
         <v>95</v>
       </c>
@@ -1574,7 +1583,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="21" spans="2:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C21" t="s">
         <v>98</v>
       </c>
@@ -1597,7 +1606,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="22" spans="2:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C22" t="s">
         <v>105</v>
       </c>
@@ -1620,7 +1629,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C23" t="s">
         <v>108</v>
       </c>
@@ -1643,7 +1652,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="24" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C24" t="s">
         <v>114</v>
       </c>
@@ -1666,7 +1675,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="25" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C25" t="s">
         <v>117</v>
       </c>
@@ -1689,7 +1698,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="26" spans="2:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="C26" t="s">
         <v>123</v>
       </c>
@@ -1712,7 +1721,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="27" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C27" t="s">
         <v>126</v>
       </c>
@@ -1735,7 +1744,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="28" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C28" t="s">
         <v>129</v>
       </c>
@@ -1758,7 +1767,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="29" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C29" t="s">
         <v>132</v>
       </c>
@@ -1781,7 +1790,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="30" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C30" t="s">
         <v>135</v>
       </c>
@@ -1804,7 +1813,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="31" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C31" t="s">
         <v>138</v>
       </c>
@@ -1827,7 +1836,10 @@
         <v>140</v>
       </c>
     </row>
-    <row r="32" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>204</v>
+      </c>
       <c r="B32" t="s">
         <v>209</v>
       </c>
@@ -1853,7 +1865,10 @@
         <v>146</v>
       </c>
     </row>
-    <row r="33" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>204</v>
+      </c>
       <c r="B33" t="s">
         <v>209</v>
       </c>
@@ -1879,7 +1894,10 @@
         <v>149</v>
       </c>
     </row>
-    <row r="34" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>204</v>
+      </c>
       <c r="B34" t="s">
         <v>209</v>
       </c>
@@ -1905,7 +1923,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="35" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C35" t="s">
         <v>154</v>
       </c>
@@ -1928,7 +1946,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="36" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C36" t="s">
         <v>160</v>
       </c>
@@ -1951,7 +1969,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="37" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C37" t="s">
         <v>163</v>
       </c>
@@ -1974,7 +1992,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="38" spans="2:9" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:9" ht="100.8" x14ac:dyDescent="0.3">
       <c r="C38" t="s">
         <v>166</v>
       </c>
@@ -1997,7 +2015,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="39" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C39" t="s">
         <v>169</v>
       </c>
@@ -2020,7 +2038,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="40" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C40" t="s">
         <v>174</v>
       </c>
@@ -2043,7 +2061,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="41" spans="2:9" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:9" ht="100.8" x14ac:dyDescent="0.3">
       <c r="C41" t="s">
         <v>177</v>
       </c>
@@ -2066,7 +2084,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="42" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C42" t="s">
         <v>180</v>
       </c>
@@ -2089,7 +2107,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="43" spans="2:9" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:9" ht="129.6" x14ac:dyDescent="0.3">
       <c r="C43" t="s">
         <v>186</v>
       </c>
@@ -2112,7 +2130,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="44" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C44" t="s">
         <v>190</v>
       </c>

</xml_diff>

<commit_message>
Atualiza dados da homologacao - 10/07/2026 14:58
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD6959C8-4363-4CBC-B6AA-45BB84C12559}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9ADC3AD7-60B2-4EF7-B32A-CF6C43F5A27D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="216">
   <si>
     <t>PENDENTE</t>
   </si>
@@ -1083,7 +1083,8 @@
   <dimension ref="A1:I44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="31.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="42.6640625" customWidth="1"/>
+    <col min="2" max="2" width="31.109375" customWidth="1"/>
     <col min="3" max="3" width="8.109375" customWidth="1"/>
     <col min="4" max="4" width="76.88671875" customWidth="1"/>
     <col min="5" max="5" width="22.5546875" bestFit="1" customWidth="1"/>
@@ -1123,12 +1124,6 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>204</v>
-      </c>
-      <c r="B2" t="s">
-        <v>201</v>
-      </c>
       <c r="C2" t="s">
         <v>10</v>
       </c>
@@ -1152,12 +1147,6 @@
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>202</v>
-      </c>
-      <c r="B3" t="s">
-        <v>203</v>
-      </c>
       <c r="C3" t="s">
         <v>16</v>
       </c>
@@ -1181,12 +1170,6 @@
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>210</v>
-      </c>
-      <c r="B4" t="s">
-        <v>201</v>
-      </c>
       <c r="C4" t="s">
         <v>23</v>
       </c>
@@ -2178,7 +2161,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{659D4760-CAB5-44F6-8F8E-F56F7A47BDF9}">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36.109375" bestFit="1" customWidth="1"/>
@@ -2187,7 +2170,7 @@
     <col min="7" max="7" width="25.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>193</v>
       </c>
@@ -2203,11 +2186,8 @@
       <c r="E1" t="s">
         <v>197</v>
       </c>
-      <c r="G1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>198</v>
       </c>
@@ -2217,27 +2197,18 @@
       <c r="C2" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="G2" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>202</v>
       </c>
-      <c r="G3" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>204</v>
       </c>
-      <c r="G4" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>206</v>
       </c>
@@ -2247,11 +2218,8 @@
       <c r="C5" t="s">
         <v>208</v>
       </c>
-      <c r="G5" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>210</v>
       </c>
@@ -2261,11 +2229,8 @@
       <c r="C6" t="s">
         <v>208</v>
       </c>
-      <c r="G6" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>213</v>
       </c>
@@ -2275,7 +2240,39 @@
       <c r="C7" t="s">
         <v>208</v>
       </c>
-      <c r="G7" t="s">
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
         <v>215</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dados da homologacao - 10/07/2026 16:57
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9ADC3AD7-60B2-4EF7-B32A-CF6C43F5A27D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{485276AB-E1F7-4A60-8A43-AAA3F8A1B426}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -161,14 +161,6 @@
     <t>CT-023</t>
   </si>
   <si>
-    <t>Atividade principal incompatível com SE
-- 1 (Agricultura, Pecuária e Outras)
-- 2 (Aquicultor)
-- 3 (Extrativista)
-- 4 (Pescador Artesanal)
-- 5 (Silvicultor)</t>
-  </si>
-  <si>
     <t>Situação</t>
   </si>
   <si>
@@ -657,9 +649,6 @@
     <t>PAT</t>
   </si>
   <si>
-    <t>Nicole Campos Otani</t>
-  </si>
-  <si>
     <t>97399884072</t>
   </si>
   <si>
@@ -669,21 +658,12 @@
     <t>Em Homologação</t>
   </si>
   <si>
-    <t>João Renato Sardinha Antunes</t>
-  </si>
-  <si>
     <t>Homologado com sucesso</t>
   </si>
   <si>
-    <t>Marcelo Caetano Figueredo Santana</t>
-  </si>
-  <si>
     <t>Reprovado</t>
   </si>
   <si>
-    <t>Graziella Sales Xavier</t>
-  </si>
-  <si>
     <t>93538413568</t>
   </si>
   <si>
@@ -693,22 +673,37 @@
     <t>Cenário cancelado</t>
   </si>
   <si>
-    <t>Gregorio Vinicius de Oliveira Bispo Dias</t>
-  </si>
-  <si>
     <t>08563524623</t>
   </si>
   <si>
     <t xml:space="preserve">Aguardando </t>
   </si>
   <si>
-    <t>Walternilson Guimarães de Souza</t>
-  </si>
-  <si>
     <t>51548569534</t>
   </si>
   <si>
     <t>Homologado com ressalvas</t>
+  </si>
+  <si>
+    <t>Nicole</t>
+  </si>
+  <si>
+    <t>João Renato</t>
+  </si>
+  <si>
+    <t>Marcelo Caetano</t>
+  </si>
+  <si>
+    <t>Graziella</t>
+  </si>
+  <si>
+    <t>Gregorio</t>
+  </si>
+  <si>
+    <t>Walternilson</t>
+  </si>
+  <si>
+    <t>Atividade principal incompatível com SE</t>
   </si>
 </sst>
 </file>
@@ -732,7 +727,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -741,7 +736,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -758,7 +759,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -766,6 +767,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1083,10 +1087,10 @@
   <dimension ref="A1:I44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="42.6640625" customWidth="1"/>
-    <col min="2" max="2" width="31.109375" customWidth="1"/>
-    <col min="3" max="3" width="8.109375" customWidth="1"/>
-    <col min="4" max="4" width="76.88671875" customWidth="1"/>
+    <col min="1" max="1" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="95.109375" customWidth="1"/>
     <col min="5" max="5" width="22.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="20.88671875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="38.44140625" bestFit="1" customWidth="1"/>
@@ -1095,31 +1099,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="5" t="s">
         <v>9</v>
       </c>
     </row>
@@ -1238,902 +1242,902 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
+        <v>211</v>
+      </c>
+      <c r="B7" t="s">
         <v>204</v>
-      </c>
-      <c r="B7" t="s">
-        <v>209</v>
       </c>
       <c r="C7" t="s">
         <v>38</v>
       </c>
       <c r="D7" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="E7" t="s">
         <v>39</v>
-      </c>
-      <c r="E7" t="s">
-        <v>40</v>
       </c>
       <c r="F7" t="s">
         <v>31</v>
       </c>
       <c r="G7" t="s">
+        <v>40</v>
+      </c>
+      <c r="H7" t="s">
         <v>41</v>
       </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>42</v>
-      </c>
-      <c r="I7" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C8" t="s">
+        <v>43</v>
+      </c>
+      <c r="D8" t="s">
         <v>44</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>45</v>
-      </c>
-      <c r="E8" t="s">
-        <v>46</v>
       </c>
       <c r="F8" t="s">
         <v>31</v>
       </c>
       <c r="G8" t="s">
+        <v>46</v>
+      </c>
+      <c r="H8" t="s">
         <v>47</v>
       </c>
-      <c r="H8" t="s">
+      <c r="I8" s="1" t="s">
         <v>48</v>
-      </c>
-      <c r="I8" s="1" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9" t="s">
         <v>50</v>
       </c>
-      <c r="D9" t="s">
-        <v>51</v>
-      </c>
       <c r="E9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F9" t="s">
         <v>0</v>
       </c>
       <c r="G9" t="s">
+        <v>51</v>
+      </c>
+      <c r="H9" t="s">
+        <v>47</v>
+      </c>
+      <c r="I9" s="1" t="s">
         <v>52</v>
-      </c>
-      <c r="H9" t="s">
-        <v>48</v>
-      </c>
-      <c r="I9" s="1" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C10" t="s">
+        <v>53</v>
+      </c>
+      <c r="D10" t="s">
         <v>54</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>55</v>
-      </c>
-      <c r="E10" t="s">
-        <v>56</v>
       </c>
       <c r="F10" t="s">
         <v>31</v>
       </c>
       <c r="G10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H10" t="s">
         <v>57</v>
       </c>
-      <c r="H10" t="s">
+      <c r="I10" s="1" t="s">
         <v>58</v>
-      </c>
-      <c r="I10" s="1" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C11" t="s">
+        <v>59</v>
+      </c>
+      <c r="D11" t="s">
         <v>60</v>
       </c>
-      <c r="D11" t="s">
-        <v>61</v>
-      </c>
       <c r="E11" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F11" t="s">
         <v>31</v>
       </c>
       <c r="G11" t="s">
+        <v>56</v>
+      </c>
+      <c r="H11" t="s">
         <v>57</v>
       </c>
-      <c r="H11" t="s">
-        <v>58</v>
-      </c>
       <c r="I11" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="C12" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="C12" t="s">
+      <c r="D12" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="E12" t="s">
+        <v>55</v>
+      </c>
+      <c r="F12" t="s">
         <v>64</v>
       </c>
-      <c r="E12" t="s">
-        <v>56</v>
-      </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
         <v>65</v>
       </c>
-      <c r="G12" t="s">
+      <c r="H12" t="s">
+        <v>57</v>
+      </c>
+      <c r="I12" s="1" t="s">
         <v>66</v>
-      </c>
-      <c r="H12" t="s">
-        <v>58</v>
-      </c>
-      <c r="I12" s="1" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C13" t="s">
+        <v>67</v>
+      </c>
+      <c r="D13" t="s">
         <v>68</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>69</v>
-      </c>
-      <c r="E13" t="s">
-        <v>70</v>
       </c>
       <c r="F13" t="s">
         <v>31</v>
       </c>
       <c r="G13" t="s">
+        <v>70</v>
+      </c>
+      <c r="H13" t="s">
         <v>71</v>
       </c>
-      <c r="H13" t="s">
+      <c r="I13" t="s">
         <v>72</v>
-      </c>
-      <c r="I13" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C14" t="s">
+        <v>73</v>
+      </c>
+      <c r="D14" t="s">
         <v>74</v>
       </c>
-      <c r="D14" t="s">
-        <v>75</v>
-      </c>
       <c r="E14" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F14" s="4" t="s">
         <v>19</v>
       </c>
       <c r="G14" t="s">
+        <v>75</v>
+      </c>
+      <c r="H14" t="s">
+        <v>71</v>
+      </c>
+      <c r="I14" t="s">
         <v>76</v>
-      </c>
-      <c r="H14" t="s">
-        <v>72</v>
-      </c>
-      <c r="I14" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C15" t="s">
+        <v>77</v>
+      </c>
+      <c r="D15" t="s">
         <v>78</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" t="s">
         <v>79</v>
       </c>
-      <c r="E15" t="s">
+      <c r="F15" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G15" t="s">
+        <v>65</v>
+      </c>
+      <c r="H15" t="s">
         <v>80</v>
       </c>
-      <c r="F15" t="s">
-        <v>65</v>
-      </c>
-      <c r="G15" t="s">
-        <v>66</v>
-      </c>
-      <c r="H15" t="s">
+      <c r="I15" t="s">
         <v>81</v>
-      </c>
-      <c r="I15" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C16" t="s">
+        <v>82</v>
+      </c>
+      <c r="D16" t="s">
         <v>83</v>
       </c>
-      <c r="D16" t="s">
-        <v>84</v>
-      </c>
       <c r="E16" t="s">
-        <v>80</v>
-      </c>
-      <c r="F16" t="s">
+        <v>79</v>
+      </c>
+      <c r="F16" s="4" t="s">
         <v>31</v>
       </c>
       <c r="G16" t="s">
         <v>32</v>
       </c>
       <c r="H16" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C17" t="s">
+        <v>85</v>
+      </c>
+      <c r="D17" t="s">
         <v>86</v>
       </c>
-      <c r="D17" t="s">
-        <v>87</v>
-      </c>
       <c r="E17" t="s">
-        <v>80</v>
-      </c>
-      <c r="F17" t="s">
+        <v>79</v>
+      </c>
+      <c r="F17" s="4" t="s">
         <v>0</v>
       </c>
       <c r="G17" t="s">
         <v>25</v>
       </c>
       <c r="H17" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="I17" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C18" t="s">
+        <v>88</v>
+      </c>
+      <c r="D18" t="s">
         <v>89</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
+        <v>79</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G18" t="s">
+        <v>65</v>
+      </c>
+      <c r="H18" t="s">
+        <v>80</v>
+      </c>
+      <c r="I18" t="s">
         <v>90</v>
-      </c>
-      <c r="E18" t="s">
-        <v>80</v>
-      </c>
-      <c r="F18" t="s">
-        <v>65</v>
-      </c>
-      <c r="G18" t="s">
-        <v>66</v>
-      </c>
-      <c r="H18" t="s">
-        <v>81</v>
-      </c>
-      <c r="I18" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C19" t="s">
+        <v>91</v>
+      </c>
+      <c r="D19" t="s">
         <v>92</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" t="s">
+        <v>79</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="G19" t="s">
+        <v>56</v>
+      </c>
+      <c r="H19" t="s">
+        <v>80</v>
+      </c>
+      <c r="I19" t="s">
         <v>93</v>
-      </c>
-      <c r="E19" t="s">
-        <v>80</v>
-      </c>
-      <c r="F19" t="s">
-        <v>31</v>
-      </c>
-      <c r="G19" t="s">
-        <v>57</v>
-      </c>
-      <c r="H19" t="s">
-        <v>81</v>
-      </c>
-      <c r="I19" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C20" t="s">
+        <v>94</v>
+      </c>
+      <c r="D20" t="s">
         <v>95</v>
       </c>
-      <c r="D20" t="s">
-        <v>96</v>
-      </c>
       <c r="E20" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F20" s="4" t="s">
         <v>19</v>
       </c>
       <c r="G20" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H20" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="I20" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C21" t="s">
+        <v>97</v>
+      </c>
+      <c r="D21" t="s">
         <v>98</v>
       </c>
-      <c r="D21" t="s">
+      <c r="E21" t="s">
         <v>99</v>
       </c>
-      <c r="E21" t="s">
+      <c r="F21" t="s">
         <v>100</v>
       </c>
-      <c r="F21" t="s">
+      <c r="G21" t="s">
         <v>101</v>
       </c>
-      <c r="G21" t="s">
+      <c r="H21" t="s">
         <v>102</v>
       </c>
-      <c r="H21" t="s">
+      <c r="I21" s="1" t="s">
         <v>103</v>
-      </c>
-      <c r="I21" s="1" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C22" t="s">
+        <v>104</v>
+      </c>
+      <c r="D22" t="s">
         <v>105</v>
       </c>
-      <c r="D22" t="s">
+      <c r="E22" t="s">
+        <v>99</v>
+      </c>
+      <c r="F22" t="s">
+        <v>64</v>
+      </c>
+      <c r="G22" t="s">
+        <v>65</v>
+      </c>
+      <c r="H22" t="s">
+        <v>102</v>
+      </c>
+      <c r="I22" s="1" t="s">
         <v>106</v>
-      </c>
-      <c r="E22" t="s">
-        <v>100</v>
-      </c>
-      <c r="F22" t="s">
-        <v>65</v>
-      </c>
-      <c r="G22" t="s">
-        <v>66</v>
-      </c>
-      <c r="H22" t="s">
-        <v>103</v>
-      </c>
-      <c r="I22" s="1" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C23" t="s">
+        <v>107</v>
+      </c>
+      <c r="D23" t="s">
         <v>108</v>
       </c>
-      <c r="D23" t="s">
+      <c r="E23" t="s">
         <v>109</v>
       </c>
-      <c r="E23" t="s">
+      <c r="F23" t="s">
+        <v>100</v>
+      </c>
+      <c r="G23" t="s">
         <v>110</v>
       </c>
-      <c r="F23" t="s">
-        <v>101</v>
-      </c>
-      <c r="G23" t="s">
+      <c r="H23" t="s">
         <v>111</v>
       </c>
-      <c r="H23" t="s">
+      <c r="I23" t="s">
         <v>112</v>
-      </c>
-      <c r="I23" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C24" t="s">
+        <v>113</v>
+      </c>
+      <c r="D24" t="s">
         <v>114</v>
       </c>
-      <c r="D24" t="s">
+      <c r="E24" t="s">
+        <v>109</v>
+      </c>
+      <c r="F24" t="s">
+        <v>64</v>
+      </c>
+      <c r="G24" t="s">
+        <v>65</v>
+      </c>
+      <c r="H24" t="s">
+        <v>111</v>
+      </c>
+      <c r="I24" t="s">
         <v>115</v>
-      </c>
-      <c r="E24" t="s">
-        <v>110</v>
-      </c>
-      <c r="F24" t="s">
-        <v>65</v>
-      </c>
-      <c r="G24" t="s">
-        <v>66</v>
-      </c>
-      <c r="H24" t="s">
-        <v>112</v>
-      </c>
-      <c r="I24" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C25" t="s">
+        <v>116</v>
+      </c>
+      <c r="D25" t="s">
         <v>117</v>
       </c>
-      <c r="D25" t="s">
+      <c r="E25" t="s">
         <v>118</v>
-      </c>
-      <c r="E25" t="s">
-        <v>119</v>
       </c>
       <c r="F25" t="s">
         <v>19</v>
       </c>
       <c r="G25" t="s">
+        <v>119</v>
+      </c>
+      <c r="H25" t="s">
         <v>120</v>
       </c>
-      <c r="H25" t="s">
+      <c r="I25" t="s">
         <v>121</v>
-      </c>
-      <c r="I25" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="26" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="C26" t="s">
+        <v>122</v>
+      </c>
+      <c r="D26" t="s">
         <v>123</v>
       </c>
-      <c r="D26" t="s">
-        <v>124</v>
-      </c>
       <c r="E26" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F26" t="s">
         <v>31</v>
       </c>
       <c r="G26" t="s">
+        <v>119</v>
+      </c>
+      <c r="H26" t="s">
         <v>120</v>
       </c>
-      <c r="H26" t="s">
-        <v>121</v>
-      </c>
       <c r="I26" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C27" t="s">
+        <v>125</v>
+      </c>
+      <c r="D27" t="s">
         <v>126</v>
       </c>
-      <c r="D27" t="s">
-        <v>127</v>
-      </c>
       <c r="E27" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F27" t="s">
         <v>31</v>
       </c>
       <c r="G27" t="s">
+        <v>119</v>
+      </c>
+      <c r="H27" t="s">
         <v>120</v>
       </c>
-      <c r="H27" t="s">
-        <v>121</v>
-      </c>
       <c r="I27" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C28" t="s">
+        <v>128</v>
+      </c>
+      <c r="D28" t="s">
         <v>129</v>
       </c>
-      <c r="D28" t="s">
-        <v>130</v>
-      </c>
       <c r="E28" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F28" t="s">
         <v>31</v>
       </c>
       <c r="G28" t="s">
+        <v>119</v>
+      </c>
+      <c r="H28" t="s">
         <v>120</v>
       </c>
-      <c r="H28" t="s">
-        <v>121</v>
-      </c>
       <c r="I28" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C29" t="s">
+        <v>131</v>
+      </c>
+      <c r="D29" t="s">
         <v>132</v>
       </c>
-      <c r="D29" t="s">
-        <v>133</v>
-      </c>
       <c r="E29" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F29" t="s">
         <v>19</v>
       </c>
       <c r="G29" t="s">
+        <v>119</v>
+      </c>
+      <c r="H29" t="s">
         <v>120</v>
       </c>
-      <c r="H29" t="s">
-        <v>121</v>
-      </c>
       <c r="I29" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C30" t="s">
+        <v>134</v>
+      </c>
+      <c r="D30" t="s">
         <v>135</v>
       </c>
-      <c r="D30" t="s">
-        <v>136</v>
-      </c>
       <c r="E30" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F30" t="s">
         <v>31</v>
       </c>
       <c r="G30" t="s">
+        <v>119</v>
+      </c>
+      <c r="H30" t="s">
         <v>120</v>
       </c>
-      <c r="H30" t="s">
-        <v>121</v>
-      </c>
       <c r="I30" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C31" t="s">
+        <v>137</v>
+      </c>
+      <c r="D31" t="s">
         <v>138</v>
       </c>
-      <c r="D31" t="s">
-        <v>139</v>
-      </c>
       <c r="E31" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F31" t="s">
         <v>31</v>
       </c>
       <c r="G31" t="s">
+        <v>119</v>
+      </c>
+      <c r="H31" t="s">
         <v>120</v>
       </c>
-      <c r="H31" t="s">
-        <v>121</v>
-      </c>
       <c r="I31" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
+        <v>211</v>
+      </c>
+      <c r="B32" t="s">
         <v>204</v>
       </c>
-      <c r="B32" t="s">
-        <v>209</v>
-      </c>
       <c r="C32" t="s">
+        <v>140</v>
+      </c>
+      <c r="D32" t="s">
         <v>141</v>
       </c>
-      <c r="D32" t="s">
+      <c r="E32" t="s">
         <v>142</v>
-      </c>
-      <c r="E32" t="s">
-        <v>143</v>
       </c>
       <c r="F32" t="s">
         <v>31</v>
       </c>
       <c r="G32" t="s">
+        <v>143</v>
+      </c>
+      <c r="H32" t="s">
         <v>144</v>
       </c>
-      <c r="H32" t="s">
+      <c r="I32" t="s">
         <v>145</v>
-      </c>
-      <c r="I32" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
+        <v>211</v>
+      </c>
+      <c r="B33" t="s">
         <v>204</v>
       </c>
-      <c r="B33" t="s">
-        <v>209</v>
-      </c>
       <c r="C33" t="s">
+        <v>146</v>
+      </c>
+      <c r="D33" t="s">
         <v>147</v>
       </c>
-      <c r="D33" t="s">
-        <v>148</v>
-      </c>
       <c r="E33" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F33" t="s">
         <v>31</v>
       </c>
       <c r="G33" t="s">
+        <v>143</v>
+      </c>
+      <c r="H33" t="s">
         <v>144</v>
       </c>
-      <c r="H33" t="s">
-        <v>145</v>
-      </c>
       <c r="I33" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
+        <v>211</v>
+      </c>
+      <c r="B34" t="s">
         <v>204</v>
       </c>
-      <c r="B34" t="s">
-        <v>209</v>
-      </c>
       <c r="C34" t="s">
+        <v>149</v>
+      </c>
+      <c r="D34" t="s">
         <v>150</v>
       </c>
-      <c r="D34" t="s">
-        <v>151</v>
-      </c>
       <c r="E34" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F34" t="s">
         <v>0</v>
       </c>
       <c r="G34" t="s">
+        <v>151</v>
+      </c>
+      <c r="H34" t="s">
+        <v>144</v>
+      </c>
+      <c r="I34" t="s">
         <v>152</v>
-      </c>
-      <c r="H34" t="s">
-        <v>145</v>
-      </c>
-      <c r="I34" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C35" t="s">
+        <v>153</v>
+      </c>
+      <c r="D35" t="s">
         <v>154</v>
       </c>
-      <c r="D35" t="s">
+      <c r="E35" t="s">
         <v>155</v>
-      </c>
-      <c r="E35" t="s">
-        <v>156</v>
       </c>
       <c r="F35" t="s">
         <v>19</v>
       </c>
       <c r="G35" t="s">
+        <v>156</v>
+      </c>
+      <c r="H35" t="s">
         <v>157</v>
       </c>
-      <c r="H35" t="s">
+      <c r="I35" t="s">
         <v>158</v>
-      </c>
-      <c r="I35" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C36" t="s">
+        <v>159</v>
+      </c>
+      <c r="D36" t="s">
         <v>160</v>
       </c>
-      <c r="D36" t="s">
-        <v>161</v>
-      </c>
       <c r="E36" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F36" t="s">
         <v>0</v>
       </c>
       <c r="G36" t="s">
+        <v>156</v>
+      </c>
+      <c r="H36" t="s">
         <v>157</v>
       </c>
-      <c r="H36" t="s">
-        <v>158</v>
-      </c>
       <c r="I36" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C37" t="s">
+        <v>162</v>
+      </c>
+      <c r="D37" t="s">
         <v>163</v>
       </c>
-      <c r="D37" t="s">
-        <v>164</v>
-      </c>
       <c r="E37" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F37" t="s">
         <v>19</v>
       </c>
       <c r="G37" t="s">
+        <v>156</v>
+      </c>
+      <c r="H37" t="s">
         <v>157</v>
       </c>
-      <c r="H37" t="s">
-        <v>158</v>
-      </c>
       <c r="I37" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="38" spans="1:9" ht="100.8" x14ac:dyDescent="0.3">
       <c r="C38" t="s">
+        <v>165</v>
+      </c>
+      <c r="D38" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="D38" s="1" t="s">
-        <v>167</v>
-      </c>
       <c r="E38" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F38" t="s">
         <v>19</v>
       </c>
       <c r="G38" t="s">
+        <v>156</v>
+      </c>
+      <c r="H38" t="s">
         <v>157</v>
       </c>
-      <c r="H38" t="s">
-        <v>158</v>
-      </c>
       <c r="I38" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C39" t="s">
+        <v>168</v>
+      </c>
+      <c r="D39" t="s">
         <v>169</v>
       </c>
-      <c r="D39" t="s">
+      <c r="E39" t="s">
         <v>170</v>
-      </c>
-      <c r="E39" t="s">
-        <v>171</v>
       </c>
       <c r="F39" t="s">
         <v>19</v>
       </c>
       <c r="G39" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H39" t="s">
+        <v>171</v>
+      </c>
+      <c r="I39" t="s">
         <v>172</v>
-      </c>
-      <c r="I39" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C40" t="s">
+        <v>173</v>
+      </c>
+      <c r="D40" t="s">
         <v>174</v>
       </c>
-      <c r="D40" t="s">
-        <v>175</v>
-      </c>
       <c r="E40" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F40" t="s">
         <v>19</v>
       </c>
       <c r="G40" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H40" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="I40" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="41" spans="1:9" ht="100.8" x14ac:dyDescent="0.3">
       <c r="C41" t="s">
+        <v>176</v>
+      </c>
+      <c r="D41" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="D41" s="1" t="s">
-        <v>178</v>
-      </c>
       <c r="E41" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F41" t="s">
         <v>19</v>
       </c>
       <c r="G41" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H41" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="I41" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C42" t="s">
+        <v>179</v>
+      </c>
+      <c r="D42" t="s">
         <v>180</v>
       </c>
-      <c r="D42" t="s">
+      <c r="E42" t="s">
         <v>181</v>
       </c>
-      <c r="E42" t="s">
+      <c r="F42" t="s">
+        <v>100</v>
+      </c>
+      <c r="G42" t="s">
         <v>182</v>
       </c>
-      <c r="F42" t="s">
-        <v>101</v>
-      </c>
-      <c r="G42" t="s">
+      <c r="H42" t="s">
         <v>183</v>
       </c>
-      <c r="H42" t="s">
+      <c r="I42" t="s">
         <v>184</v>
-      </c>
-      <c r="I42" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="43" spans="1:9" ht="129.6" x14ac:dyDescent="0.3">
       <c r="C43" t="s">
+        <v>185</v>
+      </c>
+      <c r="D43" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="D43" s="1" t="s">
+      <c r="E43" t="s">
+        <v>181</v>
+      </c>
+      <c r="F43" t="s">
+        <v>100</v>
+      </c>
+      <c r="G43" t="s">
         <v>187</v>
       </c>
-      <c r="E43" t="s">
-        <v>182</v>
-      </c>
-      <c r="F43" t="s">
-        <v>101</v>
-      </c>
-      <c r="G43" t="s">
+      <c r="H43" t="s">
+        <v>183</v>
+      </c>
+      <c r="I43" t="s">
         <v>188</v>
-      </c>
-      <c r="H43" t="s">
-        <v>184</v>
-      </c>
-      <c r="I43" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C44" t="s">
+        <v>189</v>
+      </c>
+      <c r="D44" t="s">
         <v>190</v>
       </c>
-      <c r="D44" t="s">
+      <c r="E44" t="s">
+        <v>181</v>
+      </c>
+      <c r="F44" t="s">
+        <v>64</v>
+      </c>
+      <c r="G44" t="s">
+        <v>65</v>
+      </c>
+      <c r="H44" t="s">
+        <v>183</v>
+      </c>
+      <c r="I44" t="s">
         <v>191</v>
-      </c>
-      <c r="E44" t="s">
-        <v>182</v>
-      </c>
-      <c r="F44" t="s">
-        <v>65</v>
-      </c>
-      <c r="G44" t="s">
-        <v>66</v>
-      </c>
-      <c r="H44" t="s">
-        <v>184</v>
-      </c>
-      <c r="I44" t="s">
-        <v>192</v>
       </c>
     </row>
   </sheetData>
@@ -2172,73 +2176,73 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>192</v>
+      </c>
+      <c r="B1" t="s">
         <v>193</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>194</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>195</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>196</v>
-      </c>
-      <c r="E1" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>198</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>200</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>204</v>
+        <v>211</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="C5" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="C6" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="C7" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
@@ -2248,32 +2252,32 @@
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza dados da homologacao - 13/07/2026 14:50
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{485276AB-E1F7-4A60-8A43-AAA3F8A1B426}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F2B5B69-F514-4339-8873-514D3CE269D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cenários homologação" sheetId="6" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="217">
   <si>
     <t>PENDENTE</t>
   </si>
@@ -704,6 +704,9 @@
   </si>
   <si>
     <t>Atividade principal incompatível com SE</t>
+  </si>
+  <si>
+    <t>Em Grupo</t>
   </si>
 </sst>
 </file>
@@ -1128,6 +1131,12 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>216</v>
+      </c>
+      <c r="B2" t="s">
+        <v>200</v>
+      </c>
       <c r="C2" t="s">
         <v>10</v>
       </c>
@@ -1151,6 +1160,12 @@
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>216</v>
+      </c>
+      <c r="B3" t="s">
+        <v>208</v>
+      </c>
       <c r="C3" t="s">
         <v>16</v>
       </c>
@@ -1174,6 +1189,12 @@
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>216</v>
+      </c>
+      <c r="B4" t="s">
+        <v>200</v>
+      </c>
       <c r="C4" t="s">
         <v>23</v>
       </c>
@@ -1197,6 +1218,12 @@
       </c>
     </row>
     <row r="5" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>216</v>
+      </c>
+      <c r="B5" t="s">
+        <v>208</v>
+      </c>
       <c r="C5" t="s">
         <v>28</v>
       </c>
@@ -1220,6 +1247,12 @@
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>216</v>
+      </c>
+      <c r="B6" t="s">
+        <v>201</v>
+      </c>
       <c r="C6" t="s">
         <v>35</v>
       </c>
@@ -1272,6 +1305,12 @@
       </c>
     </row>
     <row r="8" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>216</v>
+      </c>
+      <c r="B8" t="s">
+        <v>199</v>
+      </c>
       <c r="C8" t="s">
         <v>43</v>
       </c>
@@ -1979,7 +2018,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="38" spans="1:9" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:9" ht="86.4" x14ac:dyDescent="0.3">
       <c r="C38" t="s">
         <v>165</v>
       </c>
@@ -2048,7 +2087,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="41" spans="1:9" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:9" ht="86.4" x14ac:dyDescent="0.3">
       <c r="C41" t="s">
         <v>176</v>
       </c>
@@ -2094,7 +2133,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:9" ht="100.8" x14ac:dyDescent="0.3">
       <c r="C43" t="s">
         <v>185</v>
       </c>
@@ -2145,17 +2184,17 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{2155632E-300D-475D-8D13-4C5BC52FE7DF}">
+        <x14:dataValidation type="list" operator="equal" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{2BD639CC-7032-4DDA-83A6-90D67489068F}">
           <x14:formula1>
-            <xm:f>Homologadores!$A$2:$A$7</xm:f>
-          </x14:formula1>
-          <xm:sqref>A2:A44</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" operator="equal" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{9B1EBE6E-6284-4158-A391-81201344000F}">
-          <x14:formula1>
-            <xm:f>Homologadores!$G$2:$G$7</xm:f>
+            <xm:f>Homologadores!$A$18:$A$24</xm:f>
           </x14:formula1>
           <xm:sqref>B2:B44</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B6186B4D-AC17-43C9-9556-105E02C006A5}">
+          <x14:formula1>
+            <xm:f>Homologadores!$A$2:$A$8</xm:f>
+          </x14:formula1>
+          <xm:sqref>A2:A45</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2165,7 +2204,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{659D4760-CAB5-44F6-8F8E-F56F7A47BDF9}">
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36.109375" bestFit="1" customWidth="1"/>
@@ -2193,42 +2232,36 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>209</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>198</v>
+        <v>216</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>210</v>
+        <v>209</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>212</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="C5" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="C6" t="s">
         <v>203</v>
@@ -2236,47 +2269,58 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C7" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>2</v>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>214</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="C8" t="s">
+        <v>203</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>199</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
         <v>208</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dados da homologacao - 13/07/2026 16:48
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F2B5B69-F514-4339-8873-514D3CE269D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{800209F4-DBEE-499D-942D-BBC53E3E3AEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="217">
   <si>
     <t>PENDENTE</t>
   </si>
@@ -1309,7 +1309,7 @@
         <v>216</v>
       </c>
       <c r="B8" t="s">
-        <v>199</v>
+        <v>208</v>
       </c>
       <c r="C8" t="s">
         <v>43</v>
@@ -1334,6 +1334,12 @@
       </c>
     </row>
     <row r="9" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>216</v>
+      </c>
+      <c r="B9" t="s">
+        <v>201</v>
+      </c>
       <c r="C9" t="s">
         <v>49</v>
       </c>
@@ -1357,6 +1363,12 @@
       </c>
     </row>
     <row r="10" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>216</v>
+      </c>
+      <c r="B10" t="s">
+        <v>199</v>
+      </c>
       <c r="C10" t="s">
         <v>53</v>
       </c>
@@ -1380,6 +1392,12 @@
       </c>
     </row>
     <row r="11" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>216</v>
+      </c>
+      <c r="B11" t="s">
+        <v>199</v>
+      </c>
       <c r="C11" t="s">
         <v>59</v>
       </c>
@@ -1403,6 +1421,12 @@
       </c>
     </row>
     <row r="12" spans="1:9" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>209</v>
+      </c>
+      <c r="B12" t="s">
+        <v>199</v>
+      </c>
       <c r="C12" t="s">
         <v>62</v>
       </c>
@@ -1426,6 +1450,9 @@
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B13" t="s">
+        <v>206</v>
+      </c>
       <c r="C13" t="s">
         <v>67</v>
       </c>
@@ -1449,6 +1476,9 @@
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B14" t="s">
+        <v>206</v>
+      </c>
       <c r="C14" t="s">
         <v>73</v>
       </c>
@@ -1472,6 +1502,12 @@
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>212</v>
+      </c>
+      <c r="B15" t="s">
+        <v>199</v>
+      </c>
       <c r="C15" t="s">
         <v>77</v>
       </c>
@@ -1495,6 +1531,9 @@
       </c>
     </row>
     <row r="16" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B16" t="s">
+        <v>206</v>
+      </c>
       <c r="C16" t="s">
         <v>82</v>
       </c>
@@ -1518,6 +1557,9 @@
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B17" t="s">
+        <v>206</v>
+      </c>
       <c r="C17" t="s">
         <v>85</v>
       </c>
@@ -1541,6 +1583,9 @@
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B18" t="s">
+        <v>206</v>
+      </c>
       <c r="C18" t="s">
         <v>88</v>
       </c>
@@ -1564,6 +1609,9 @@
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B19" t="s">
+        <v>206</v>
+      </c>
       <c r="C19" t="s">
         <v>91</v>
       </c>
@@ -1587,6 +1635,9 @@
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B20" t="s">
+        <v>206</v>
+      </c>
       <c r="C20" t="s">
         <v>94</v>
       </c>
@@ -1610,6 +1661,9 @@
       </c>
     </row>
     <row r="21" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B21" t="s">
+        <v>206</v>
+      </c>
       <c r="C21" t="s">
         <v>97</v>
       </c>
@@ -1633,6 +1687,9 @@
       </c>
     </row>
     <row r="22" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B22" t="s">
+        <v>206</v>
+      </c>
       <c r="C22" t="s">
         <v>104</v>
       </c>
@@ -1656,6 +1713,9 @@
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B23" t="s">
+        <v>206</v>
+      </c>
       <c r="C23" t="s">
         <v>107</v>
       </c>
@@ -1679,6 +1739,9 @@
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B24" t="s">
+        <v>206</v>
+      </c>
       <c r="C24" t="s">
         <v>113</v>
       </c>
@@ -1702,6 +1765,9 @@
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B25" t="s">
+        <v>206</v>
+      </c>
       <c r="C25" t="s">
         <v>116</v>
       </c>
@@ -1725,6 +1791,9 @@
       </c>
     </row>
     <row r="26" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B26" t="s">
+        <v>206</v>
+      </c>
       <c r="C26" t="s">
         <v>122</v>
       </c>
@@ -1748,6 +1817,9 @@
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B27" t="s">
+        <v>206</v>
+      </c>
       <c r="C27" t="s">
         <v>125</v>
       </c>
@@ -1771,6 +1843,9 @@
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B28" t="s">
+        <v>206</v>
+      </c>
       <c r="C28" t="s">
         <v>128</v>
       </c>
@@ -1794,6 +1869,9 @@
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B29" t="s">
+        <v>206</v>
+      </c>
       <c r="C29" t="s">
         <v>131</v>
       </c>
@@ -1817,6 +1895,9 @@
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B30" t="s">
+        <v>206</v>
+      </c>
       <c r="C30" t="s">
         <v>134</v>
       </c>
@@ -1840,6 +1921,9 @@
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B31" t="s">
+        <v>206</v>
+      </c>
       <c r="C31" t="s">
         <v>137</v>
       </c>
@@ -1950,6 +2034,9 @@
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B35" t="s">
+        <v>206</v>
+      </c>
       <c r="C35" t="s">
         <v>153</v>
       </c>
@@ -1973,6 +2060,9 @@
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B36" t="s">
+        <v>206</v>
+      </c>
       <c r="C36" t="s">
         <v>159</v>
       </c>
@@ -1996,6 +2086,9 @@
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B37" t="s">
+        <v>206</v>
+      </c>
       <c r="C37" t="s">
         <v>162</v>
       </c>
@@ -2019,6 +2112,9 @@
       </c>
     </row>
     <row r="38" spans="1:9" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="B38" t="s">
+        <v>206</v>
+      </c>
       <c r="C38" t="s">
         <v>165</v>
       </c>
@@ -2065,6 +2161,9 @@
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B40" t="s">
+        <v>206</v>
+      </c>
       <c r="C40" t="s">
         <v>173</v>
       </c>
@@ -2088,6 +2187,9 @@
       </c>
     </row>
     <row r="41" spans="1:9" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="B41" t="s">
+        <v>206</v>
+      </c>
       <c r="C41" t="s">
         <v>176</v>
       </c>
@@ -2111,6 +2213,9 @@
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B42" t="s">
+        <v>206</v>
+      </c>
       <c r="C42" t="s">
         <v>179</v>
       </c>
@@ -2134,6 +2239,9 @@
       </c>
     </row>
     <row r="43" spans="1:9" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="B43" t="s">
+        <v>206</v>
+      </c>
       <c r="C43" t="s">
         <v>185</v>
       </c>
@@ -2157,6 +2265,9 @@
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B44" t="s">
+        <v>206</v>
+      </c>
       <c r="C44" t="s">
         <v>189</v>
       </c>

</xml_diff>

<commit_message>
Atualiza dados da homologacao - 13/07/2026 17:14
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{800209F4-DBEE-499D-942D-BBC53E3E3AEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3AB0B10-DD5D-44FE-9DC0-29E5C0758FB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="367" uniqueCount="217">
   <si>
     <t>PENDENTE</t>
   </si>
@@ -1450,9 +1450,6 @@
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B13" t="s">
-        <v>206</v>
-      </c>
       <c r="C13" t="s">
         <v>67</v>
       </c>
@@ -1476,9 +1473,6 @@
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B14" t="s">
-        <v>206</v>
-      </c>
       <c r="C14" t="s">
         <v>73</v>
       </c>
@@ -1531,9 +1525,6 @@
       </c>
     </row>
     <row r="16" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B16" t="s">
-        <v>206</v>
-      </c>
       <c r="C16" t="s">
         <v>82</v>
       </c>
@@ -1557,9 +1548,6 @@
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B17" t="s">
-        <v>206</v>
-      </c>
       <c r="C17" t="s">
         <v>85</v>
       </c>
@@ -1583,9 +1571,6 @@
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B18" t="s">
-        <v>206</v>
-      </c>
       <c r="C18" t="s">
         <v>88</v>
       </c>
@@ -1609,9 +1594,6 @@
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B19" t="s">
-        <v>206</v>
-      </c>
       <c r="C19" t="s">
         <v>91</v>
       </c>
@@ -1635,9 +1617,6 @@
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B20" t="s">
-        <v>206</v>
-      </c>
       <c r="C20" t="s">
         <v>94</v>
       </c>
@@ -1661,9 +1640,6 @@
       </c>
     </row>
     <row r="21" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B21" t="s">
-        <v>206</v>
-      </c>
       <c r="C21" t="s">
         <v>97</v>
       </c>
@@ -1687,9 +1663,6 @@
       </c>
     </row>
     <row r="22" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B22" t="s">
-        <v>206</v>
-      </c>
       <c r="C22" t="s">
         <v>104</v>
       </c>
@@ -1713,9 +1686,6 @@
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B23" t="s">
-        <v>206</v>
-      </c>
       <c r="C23" t="s">
         <v>107</v>
       </c>
@@ -1739,9 +1709,6 @@
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B24" t="s">
-        <v>206</v>
-      </c>
       <c r="C24" t="s">
         <v>113</v>
       </c>
@@ -1765,9 +1732,6 @@
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B25" t="s">
-        <v>206</v>
-      </c>
       <c r="C25" t="s">
         <v>116</v>
       </c>
@@ -1791,9 +1755,6 @@
       </c>
     </row>
     <row r="26" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B26" t="s">
-        <v>206</v>
-      </c>
       <c r="C26" t="s">
         <v>122</v>
       </c>
@@ -1817,9 +1778,6 @@
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B27" t="s">
-        <v>206</v>
-      </c>
       <c r="C27" t="s">
         <v>125</v>
       </c>
@@ -1843,9 +1801,6 @@
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B28" t="s">
-        <v>206</v>
-      </c>
       <c r="C28" t="s">
         <v>128</v>
       </c>
@@ -1869,9 +1824,6 @@
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B29" t="s">
-        <v>206</v>
-      </c>
       <c r="C29" t="s">
         <v>131</v>
       </c>
@@ -1895,9 +1847,6 @@
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B30" t="s">
-        <v>206</v>
-      </c>
       <c r="C30" t="s">
         <v>134</v>
       </c>
@@ -1921,9 +1870,6 @@
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B31" t="s">
-        <v>206</v>
-      </c>
       <c r="C31" t="s">
         <v>137</v>
       </c>
@@ -2034,9 +1980,6 @@
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B35" t="s">
-        <v>206</v>
-      </c>
       <c r="C35" t="s">
         <v>153</v>
       </c>
@@ -2060,9 +2003,6 @@
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B36" t="s">
-        <v>206</v>
-      </c>
       <c r="C36" t="s">
         <v>159</v>
       </c>
@@ -2086,9 +2026,6 @@
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B37" t="s">
-        <v>206</v>
-      </c>
       <c r="C37" t="s">
         <v>162</v>
       </c>
@@ -2112,9 +2049,6 @@
       </c>
     </row>
     <row r="38" spans="1:9" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B38" t="s">
-        <v>206</v>
-      </c>
       <c r="C38" t="s">
         <v>165</v>
       </c>
@@ -2161,9 +2095,6 @@
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B40" t="s">
-        <v>206</v>
-      </c>
       <c r="C40" t="s">
         <v>173</v>
       </c>
@@ -2187,9 +2118,6 @@
       </c>
     </row>
     <row r="41" spans="1:9" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B41" t="s">
-        <v>206</v>
-      </c>
       <c r="C41" t="s">
         <v>176</v>
       </c>
@@ -2213,9 +2141,6 @@
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B42" t="s">
-        <v>206</v>
-      </c>
       <c r="C42" t="s">
         <v>179</v>
       </c>
@@ -2239,9 +2164,6 @@
       </c>
     </row>
     <row r="43" spans="1:9" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="B43" t="s">
-        <v>206</v>
-      </c>
       <c r="C43" t="s">
         <v>185</v>
       </c>
@@ -2265,9 +2187,6 @@
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B44" t="s">
-        <v>206</v>
-      </c>
       <c r="C44" t="s">
         <v>189</v>
       </c>

</xml_diff>

<commit_message>
Atualiza dados da homologacao - 13/07/2026 17:58
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3AB0B10-DD5D-44FE-9DC0-29E5C0758FB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFF6A688-A05F-480B-95C3-5F35201C7BB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="367" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="217">
   <si>
     <t>PENDENTE</t>
   </si>
@@ -1091,7 +1091,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.88671875" customWidth="1"/>
     <col min="3" max="3" width="18" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="95.109375" customWidth="1"/>
     <col min="5" max="5" width="22.5546875" bestFit="1" customWidth="1"/>
@@ -1366,9 +1366,6 @@
       <c r="A10" t="s">
         <v>216</v>
       </c>
-      <c r="B10" t="s">
-        <v>199</v>
-      </c>
       <c r="C10" t="s">
         <v>53</v>
       </c>
@@ -1425,7 +1422,7 @@
         <v>209</v>
       </c>
       <c r="B12" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C12" t="s">
         <v>62</v>
@@ -1450,6 +1447,12 @@
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>209</v>
+      </c>
+      <c r="B13" t="s">
+        <v>199</v>
+      </c>
       <c r="C13" t="s">
         <v>67</v>
       </c>
@@ -1473,6 +1476,12 @@
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>211</v>
+      </c>
+      <c r="B14" t="s">
+        <v>204</v>
+      </c>
       <c r="C14" t="s">
         <v>73</v>
       </c>
@@ -1500,7 +1509,7 @@
         <v>212</v>
       </c>
       <c r="B15" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C15" t="s">
         <v>77</v>
@@ -1525,6 +1534,12 @@
       </c>
     </row>
     <row r="16" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>214</v>
+      </c>
+      <c r="B16" t="s">
+        <v>208</v>
+      </c>
       <c r="C16" t="s">
         <v>82</v>
       </c>
@@ -1548,6 +1563,12 @@
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>216</v>
+      </c>
+      <c r="B17" t="s">
+        <v>201</v>
+      </c>
       <c r="C17" t="s">
         <v>85</v>
       </c>
@@ -1571,6 +1592,12 @@
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>216</v>
+      </c>
+      <c r="B18" t="s">
+        <v>201</v>
+      </c>
       <c r="C18" t="s">
         <v>88</v>
       </c>
@@ -1594,6 +1621,12 @@
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>216</v>
+      </c>
+      <c r="B19" t="s">
+        <v>199</v>
+      </c>
       <c r="C19" t="s">
         <v>91</v>
       </c>

</xml_diff>

<commit_message>
Atualiza dados da homologacao - 14/07/2026 10:03
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFF6A688-A05F-480B-95C3-5F35201C7BB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDC06A45-1AE7-4471-97A9-672ADB71028A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="219">
   <si>
     <t>PENDENTE</t>
   </si>
@@ -707,6 +707,12 @@
   </si>
   <si>
     <t>Em Grupo</t>
+  </si>
+  <si>
+    <t>Disponivel para Reteste</t>
+  </si>
+  <si>
+    <t>Em Reteste</t>
   </si>
 </sst>
 </file>
@@ -1164,7 +1170,7 @@
         <v>216</v>
       </c>
       <c r="B3" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C3" t="s">
         <v>16</v>
@@ -1222,7 +1228,7 @@
         <v>216</v>
       </c>
       <c r="B5" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C5" t="s">
         <v>28</v>
@@ -1251,7 +1257,7 @@
         <v>216</v>
       </c>
       <c r="B6" t="s">
-        <v>201</v>
+        <v>218</v>
       </c>
       <c r="C6" t="s">
         <v>35</v>
@@ -1309,7 +1315,7 @@
         <v>216</v>
       </c>
       <c r="B8" t="s">
-        <v>208</v>
+        <v>217</v>
       </c>
       <c r="C8" t="s">
         <v>43</v>
@@ -1363,9 +1369,6 @@
       </c>
     </row>
     <row r="10" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>216</v>
-      </c>
       <c r="C10" t="s">
         <v>53</v>
       </c>
@@ -1509,7 +1512,7 @@
         <v>212</v>
       </c>
       <c r="B15" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C15" t="s">
         <v>77</v>
@@ -2082,6 +2085,12 @@
       </c>
     </row>
     <row r="38" spans="1:9" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>211</v>
+      </c>
+      <c r="B38" t="s">
+        <v>204</v>
+      </c>
       <c r="C38" t="s">
         <v>165</v>
       </c>
@@ -2105,6 +2114,12 @@
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>211</v>
+      </c>
+      <c r="B39" t="s">
+        <v>204</v>
+      </c>
       <c r="C39" t="s">
         <v>168</v>
       </c>
@@ -2128,6 +2143,12 @@
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>211</v>
+      </c>
+      <c r="B40" t="s">
+        <v>204</v>
+      </c>
       <c r="C40" t="s">
         <v>173</v>
       </c>
@@ -2249,7 +2270,7 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
         <x14:dataValidation type="list" operator="equal" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{2BD639CC-7032-4DDA-83A6-90D67489068F}">
           <x14:formula1>
-            <xm:f>Homologadores!$A$18:$A$24</xm:f>
+            <xm:f>Homologadores!$A$18:$A$26</xm:f>
           </x14:formula1>
           <xm:sqref>B2:B44</xm:sqref>
         </x14:dataValidation>
@@ -2267,7 +2288,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{659D4760-CAB5-44F6-8F8E-F56F7A47BDF9}">
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36.109375" bestFit="1" customWidth="1"/>
@@ -2364,26 +2385,36 @@
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>200</v>
+        <v>217</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>201</v>
+        <v>218</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
         <v>208</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dados da homologacao - 14/07/2026 11:47
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDC06A45-1AE7-4471-97A9-672ADB71028A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{724140C8-2A9B-495F-83DB-4338D4C1249B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1451,7 +1451,7 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>209</v>
+        <v>216</v>
       </c>
       <c r="B13" t="s">
         <v>199</v>
@@ -1541,7 +1541,7 @@
         <v>214</v>
       </c>
       <c r="B16" t="s">
-        <v>208</v>
+        <v>217</v>
       </c>
       <c r="C16" t="s">
         <v>82</v>

</xml_diff>

<commit_message>
Atualiza dados da homologacao - 14/07/2026 12:37
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{724140C8-2A9B-495F-83DB-4338D4C1249B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D73357FC-A8CF-4581-AFA9-777C99D2CCBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1257,7 +1257,7 @@
         <v>216</v>
       </c>
       <c r="B6" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C6" t="s">
         <v>35</v>
@@ -1512,7 +1512,7 @@
         <v>212</v>
       </c>
       <c r="B15" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C15" t="s">
         <v>77</v>
@@ -1570,7 +1570,7 @@
         <v>216</v>
       </c>
       <c r="B17" t="s">
-        <v>201</v>
+        <v>217</v>
       </c>
       <c r="C17" t="s">
         <v>85</v>
@@ -1628,7 +1628,7 @@
         <v>216</v>
       </c>
       <c r="B19" t="s">
-        <v>199</v>
+        <v>217</v>
       </c>
       <c r="C19" t="s">
         <v>91</v>

</xml_diff>

<commit_message>
Atualiza dados da homologacao - 14/07/2026 14:36
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D73357FC-A8CF-4581-AFA9-777C99D2CCBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30A7D4DC-2371-43C6-840F-56E5FCA017BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1315,7 +1315,7 @@
         <v>216</v>
       </c>
       <c r="B8" t="s">
-        <v>217</v>
+        <v>201</v>
       </c>
       <c r="C8" t="s">
         <v>43</v>
@@ -1396,7 +1396,7 @@
         <v>216</v>
       </c>
       <c r="B11" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C11" t="s">
         <v>59</v>
@@ -1454,7 +1454,7 @@
         <v>216</v>
       </c>
       <c r="B13" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C13" t="s">
         <v>67</v>
@@ -1541,7 +1541,7 @@
         <v>214</v>
       </c>
       <c r="B16" t="s">
-        <v>217</v>
+        <v>200</v>
       </c>
       <c r="C16" t="s">
         <v>82</v>

</xml_diff>

<commit_message>
Atualiza dados da homologacao - 14/07/2026 17:33
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30A7D4DC-2371-43C6-840F-56E5FCA017BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FE691E5-6165-4794-894F-5007D2D8A3B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="219">
   <si>
     <t>PENDENTE</t>
   </si>
@@ -1570,7 +1570,7 @@
         <v>216</v>
       </c>
       <c r="B17" t="s">
-        <v>217</v>
+        <v>200</v>
       </c>
       <c r="C17" t="s">
         <v>85</v>
@@ -1653,6 +1653,12 @@
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>216</v>
+      </c>
+      <c r="B20" t="s">
+        <v>199</v>
+      </c>
       <c r="C20" t="s">
         <v>94</v>
       </c>
@@ -1699,6 +1705,12 @@
       </c>
     </row>
     <row r="22" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>216</v>
+      </c>
+      <c r="B22" t="s">
+        <v>199</v>
+      </c>
       <c r="C22" t="s">
         <v>104</v>
       </c>
@@ -1722,6 +1734,12 @@
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>216</v>
+      </c>
+      <c r="B23" t="s">
+        <v>199</v>
+      </c>
       <c r="C23" t="s">
         <v>107</v>
       </c>

</xml_diff>

<commit_message>
Atualiza dados da homologacao - 15/07/2026 10:03
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FE691E5-6165-4794-894F-5007D2D8A3B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22B66D67-109C-4AE8-9EEB-41A0DC2712ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="219">
   <si>
     <t>PENDENTE</t>
   </si>
@@ -1257,7 +1257,7 @@
         <v>216</v>
       </c>
       <c r="B6" t="s">
-        <v>217</v>
+        <v>199</v>
       </c>
       <c r="C6" t="s">
         <v>35</v>
@@ -1454,7 +1454,7 @@
         <v>216</v>
       </c>
       <c r="B13" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C13" t="s">
         <v>67</v>
@@ -1628,7 +1628,7 @@
         <v>216</v>
       </c>
       <c r="B19" t="s">
-        <v>217</v>
+        <v>201</v>
       </c>
       <c r="C19" t="s">
         <v>91</v>
@@ -1657,7 +1657,7 @@
         <v>216</v>
       </c>
       <c r="B20" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C20" t="s">
         <v>94</v>
@@ -1705,12 +1705,6 @@
       </c>
     </row>
     <row r="22" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>216</v>
-      </c>
-      <c r="B22" t="s">
-        <v>199</v>
-      </c>
       <c r="C22" t="s">
         <v>104</v>
       </c>
@@ -1738,7 +1732,7 @@
         <v>216</v>
       </c>
       <c r="B23" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C23" t="s">
         <v>107</v>
@@ -1763,6 +1757,12 @@
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>216</v>
+      </c>
+      <c r="B24" t="s">
+        <v>199</v>
+      </c>
       <c r="C24" t="s">
         <v>113</v>
       </c>
@@ -1786,6 +1786,12 @@
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>216</v>
+      </c>
+      <c r="B25" t="s">
+        <v>199</v>
+      </c>
       <c r="C25" t="s">
         <v>116</v>
       </c>

</xml_diff>

<commit_message>
Atualiza dados da homologacao - 15/07/2026 15:17
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22B66D67-109C-4AE8-9EEB-41A0DC2712ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB376616-D60E-40C8-9A0E-2376724C9AE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="219">
   <si>
     <t>PENDENTE</t>
   </si>
@@ -1315,7 +1315,7 @@
         <v>216</v>
       </c>
       <c r="B8" t="s">
-        <v>201</v>
+        <v>217</v>
       </c>
       <c r="C8" t="s">
         <v>43</v>
@@ -1344,7 +1344,7 @@
         <v>216</v>
       </c>
       <c r="B9" t="s">
-        <v>201</v>
+        <v>217</v>
       </c>
       <c r="C9" t="s">
         <v>49</v>
@@ -1396,7 +1396,7 @@
         <v>216</v>
       </c>
       <c r="B11" t="s">
-        <v>201</v>
+        <v>217</v>
       </c>
       <c r="C11" t="s">
         <v>59</v>
@@ -1425,7 +1425,7 @@
         <v>209</v>
       </c>
       <c r="B12" t="s">
-        <v>201</v>
+        <v>217</v>
       </c>
       <c r="C12" t="s">
         <v>62</v>
@@ -1454,7 +1454,7 @@
         <v>216</v>
       </c>
       <c r="B13" t="s">
-        <v>199</v>
+        <v>217</v>
       </c>
       <c r="C13" t="s">
         <v>67</v>
@@ -1512,7 +1512,7 @@
         <v>212</v>
       </c>
       <c r="B15" t="s">
-        <v>201</v>
+        <v>217</v>
       </c>
       <c r="C15" t="s">
         <v>77</v>
@@ -1599,7 +1599,7 @@
         <v>216</v>
       </c>
       <c r="B18" t="s">
-        <v>201</v>
+        <v>217</v>
       </c>
       <c r="C18" t="s">
         <v>88</v>
@@ -1628,7 +1628,7 @@
         <v>216</v>
       </c>
       <c r="B19" t="s">
-        <v>201</v>
+        <v>217</v>
       </c>
       <c r="C19" t="s">
         <v>91</v>
@@ -1705,6 +1705,12 @@
       </c>
     </row>
     <row r="22" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>216</v>
+      </c>
+      <c r="B22" t="s">
+        <v>217</v>
+      </c>
       <c r="C22" t="s">
         <v>104</v>
       </c>
@@ -1761,7 +1767,7 @@
         <v>216</v>
       </c>
       <c r="B24" t="s">
-        <v>199</v>
+        <v>217</v>
       </c>
       <c r="C24" t="s">
         <v>113</v>
@@ -1790,7 +1796,7 @@
         <v>216</v>
       </c>
       <c r="B25" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C25" t="s">
         <v>116</v>
@@ -1815,6 +1821,12 @@
       </c>
     </row>
     <row r="26" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>216</v>
+      </c>
+      <c r="B26" t="s">
+        <v>199</v>
+      </c>
       <c r="C26" t="s">
         <v>122</v>
       </c>
@@ -1838,6 +1850,12 @@
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>216</v>
+      </c>
+      <c r="B27" t="s">
+        <v>199</v>
+      </c>
       <c r="C27" t="s">
         <v>125</v>
       </c>

</xml_diff>

<commit_message>
Atualiza dados da homologacao - 15/07/2026 16:58
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB376616-D60E-40C8-9A0E-2376724C9AE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87CDBD6F-1168-4DDE-8109-2E28C9311C3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cenários homologação" sheetId="6" r:id="rId1"/>
@@ -1257,7 +1257,7 @@
         <v>216</v>
       </c>
       <c r="B6" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C6" t="s">
         <v>35</v>
@@ -1315,7 +1315,7 @@
         <v>216</v>
       </c>
       <c r="B8" t="s">
-        <v>217</v>
+        <v>199</v>
       </c>
       <c r="C8" t="s">
         <v>43</v>
@@ -1541,7 +1541,7 @@
         <v>214</v>
       </c>
       <c r="B16" t="s">
-        <v>200</v>
+        <v>217</v>
       </c>
       <c r="C16" t="s">
         <v>82</v>

</xml_diff>

<commit_message>
Atualiza dados da homologacao - 16/07/2026 17:13
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87CDBD6F-1168-4DDE-8109-2E28C9311C3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91C0B5AA-3177-47F8-9BBE-8B4EF88F1884}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cenários homologação" sheetId="6" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="220">
   <si>
     <t>PENDENTE</t>
   </si>
@@ -713,6 +713,9 @@
   </si>
   <si>
     <t>Em Reteste</t>
+  </si>
+  <si>
+    <t>Janaina</t>
   </si>
 </sst>
 </file>
@@ -1315,7 +1318,7 @@
         <v>216</v>
       </c>
       <c r="B8" t="s">
-        <v>199</v>
+        <v>218</v>
       </c>
       <c r="C8" t="s">
         <v>43</v>
@@ -1344,7 +1347,7 @@
         <v>216</v>
       </c>
       <c r="B9" t="s">
-        <v>217</v>
+        <v>201</v>
       </c>
       <c r="C9" t="s">
         <v>49</v>
@@ -1369,6 +1372,12 @@
       </c>
     </row>
     <row r="10" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>212</v>
+      </c>
+      <c r="B10" t="s">
+        <v>201</v>
+      </c>
       <c r="C10" t="s">
         <v>53</v>
       </c>
@@ -1393,10 +1402,10 @@
     </row>
     <row r="11" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="B11" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="C11" t="s">
         <v>59</v>
@@ -1425,7 +1434,7 @@
         <v>209</v>
       </c>
       <c r="B12" t="s">
-        <v>217</v>
+        <v>201</v>
       </c>
       <c r="C12" t="s">
         <v>62</v>
@@ -1451,10 +1460,10 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B13" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="C13" t="s">
         <v>67</v>
@@ -1512,7 +1521,7 @@
         <v>212</v>
       </c>
       <c r="B15" t="s">
-        <v>217</v>
+        <v>200</v>
       </c>
       <c r="C15" t="s">
         <v>77</v>
@@ -1541,7 +1550,7 @@
         <v>214</v>
       </c>
       <c r="B16" t="s">
-        <v>217</v>
+        <v>200</v>
       </c>
       <c r="C16" t="s">
         <v>82</v>
@@ -1599,7 +1608,7 @@
         <v>216</v>
       </c>
       <c r="B18" t="s">
-        <v>217</v>
+        <v>201</v>
       </c>
       <c r="C18" t="s">
         <v>88</v>
@@ -1628,7 +1637,7 @@
         <v>216</v>
       </c>
       <c r="B19" t="s">
-        <v>217</v>
+        <v>201</v>
       </c>
       <c r="C19" t="s">
         <v>91</v>
@@ -1682,6 +1691,12 @@
       </c>
     </row>
     <row r="21" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>216</v>
+      </c>
+      <c r="B21" t="s">
+        <v>200</v>
+      </c>
       <c r="C21" t="s">
         <v>97</v>
       </c>
@@ -1709,7 +1724,7 @@
         <v>216</v>
       </c>
       <c r="B22" t="s">
-        <v>217</v>
+        <v>201</v>
       </c>
       <c r="C22" t="s">
         <v>104</v>
@@ -1767,7 +1782,7 @@
         <v>216</v>
       </c>
       <c r="B24" t="s">
-        <v>217</v>
+        <v>201</v>
       </c>
       <c r="C24" t="s">
         <v>113</v>
@@ -2283,6 +2298,12 @@
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>209</v>
+      </c>
+      <c r="B44" t="s">
+        <v>208</v>
+      </c>
       <c r="C44" t="s">
         <v>189</v>
       </c>
@@ -2312,13 +2333,13 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
         <x14:dataValidation type="list" operator="equal" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{2BD639CC-7032-4DDA-83A6-90D67489068F}">
           <x14:formula1>
-            <xm:f>Homologadores!$A$18:$A$26</xm:f>
+            <xm:f>Homologadores!$A$19:$A$27</xm:f>
           </x14:formula1>
           <xm:sqref>B2:B44</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B6186B4D-AC17-43C9-9556-105E02C006A5}">
           <x14:formula1>
-            <xm:f>Homologadores!$A$2:$A$8</xm:f>
+            <xm:f>Homologadores!$A$2:$A$9</xm:f>
           </x14:formula1>
           <xm:sqref>A2:A45</xm:sqref>
         </x14:dataValidation>
@@ -2330,7 +2351,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{659D4760-CAB5-44F6-8F8E-F56F7A47BDF9}">
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36.109375" bestFit="1" customWidth="1"/>
@@ -2374,31 +2395,27 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>210</v>
-      </c>
+        <v>219</v>
+      </c>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>212</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="C6" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="C7" t="s">
         <v>203</v>
@@ -2406,57 +2423,68 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C8" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>2</v>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>214</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="C9" t="s">
+        <v>203</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>199</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>217</v>
+        <v>199</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>200</v>
+        <v>218</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
         <v>208</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dados da homologacao - 17/07/2026 15:27
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91C0B5AA-3177-47F8-9BBE-8B4EF88F1884}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F44F53D6-1A49-443C-B7EA-7EADD3D33334}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="221">
   <si>
     <t>PENDENTE</t>
   </si>
@@ -716,6 +716,9 @@
   </si>
   <si>
     <t>Janaina</t>
+  </si>
+  <si>
+    <t>Aguadando cenários</t>
   </si>
 </sst>
 </file>
@@ -739,7 +742,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -758,6 +761,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -771,7 +786,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -781,6 +796,14 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1101,13 +1124,13 @@
   <cols>
     <col min="1" max="1" width="15.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="27.88671875" customWidth="1"/>
-    <col min="3" max="3" width="18" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="95.109375" customWidth="1"/>
+    <col min="3" max="3" width="9" customWidth="1"/>
+    <col min="4" max="4" width="40.33203125" customWidth="1"/>
     <col min="5" max="5" width="22.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="20.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="38.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="32.109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="107.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.77734375" customWidth="1"/>
+    <col min="8" max="8" width="18.44140625" customWidth="1"/>
+    <col min="9" max="9" width="35" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.3">
@@ -1140,205 +1163,205 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" s="6" t="s">
         <v>216</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="I2" s="7" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="A3" s="6" t="s">
         <v>216</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="I3" t="s">
+      <c r="I3" s="6" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="A4" s="6" t="s">
         <v>216</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="H4" t="s">
+      <c r="H4" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" s="6" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="A5" s="6" t="s">
         <v>216</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="H5" t="s">
+      <c r="H5" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="I5" s="7" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="A6" s="6" t="s">
         <v>216</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="H6" t="s">
+      <c r="H6" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I6" s="6" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="A7" s="8" t="s">
         <v>211</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="8" t="s">
         <v>204</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" s="9" t="s">
         <v>215</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="H7" t="s">
+      <c r="H7" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="I7" t="s">
+      <c r="I7" s="8" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+      <c r="A8" s="6" t="s">
         <v>216</v>
       </c>
-      <c r="B8" t="s">
-        <v>218</v>
-      </c>
-      <c r="C8" t="s">
+      <c r="B8" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="C8" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="G8" t="s">
+      <c r="G8" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="H8" t="s">
+      <c r="H8" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="I8" s="1" t="s">
+      <c r="I8" s="7" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1347,7 +1370,7 @@
         <v>216</v>
       </c>
       <c r="B9" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="C9" t="s">
         <v>49</v>
@@ -1405,7 +1428,7 @@
         <v>209</v>
       </c>
       <c r="B11" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="C11" t="s">
         <v>59</v>
@@ -1434,7 +1457,7 @@
         <v>209</v>
       </c>
       <c r="B12" t="s">
-        <v>201</v>
+        <v>220</v>
       </c>
       <c r="C12" t="s">
         <v>62</v>
@@ -1463,7 +1486,7 @@
         <v>214</v>
       </c>
       <c r="B13" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="C13" t="s">
         <v>67</v>
@@ -1488,118 +1511,118 @@
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
+      <c r="A14" s="8" t="s">
         <v>211</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="8" t="s">
         <v>204</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="F14" s="4" t="s">
+      <c r="F14" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="G14" t="s">
+      <c r="G14" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="H14" t="s">
+      <c r="H14" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="I14" t="s">
+      <c r="I14" s="8" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
+      <c r="A15" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="F15" s="4" t="s">
+      <c r="F15" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="G15" t="s">
+      <c r="G15" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="H15" t="s">
+      <c r="H15" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="I15" t="s">
+      <c r="I15" s="6" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
+      <c r="A16" s="6" t="s">
         <v>214</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="F16" s="4" t="s">
+      <c r="F16" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="G16" t="s">
+      <c r="G16" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="H16" t="s">
+      <c r="H16" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="I16" s="1" t="s">
+      <c r="I16" s="7" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
+      <c r="A17" s="6" t="s">
         <v>216</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E17" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="F17" s="4" t="s">
+      <c r="F17" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="G17" t="s">
+      <c r="G17" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="H17" t="s">
+      <c r="H17" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="I17" t="s">
+      <c r="I17" s="6" t="s">
         <v>87</v>
       </c>
     </row>
@@ -1691,31 +1714,31 @@
       </c>
     </row>
     <row r="21" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
+      <c r="A21" s="6" t="s">
         <v>216</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D21" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="E21" t="s">
+      <c r="E21" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="F21" t="s">
+      <c r="F21" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="G21" t="s">
+      <c r="G21" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="H21" t="s">
+      <c r="H21" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="I21" s="1" t="s">
+      <c r="I21" s="7" t="s">
         <v>103</v>
       </c>
     </row>
@@ -1749,31 +1772,31 @@
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
+      <c r="A23" s="6" t="s">
         <v>216</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D23" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="E23" t="s">
+      <c r="E23" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="F23" t="s">
+      <c r="F23" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="H23" t="s">
+      <c r="H23" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" s="6" t="s">
         <v>112</v>
       </c>
     </row>
@@ -1840,7 +1863,7 @@
         <v>216</v>
       </c>
       <c r="B26" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C26" t="s">
         <v>122</v>
@@ -1869,7 +1892,7 @@
         <v>216</v>
       </c>
       <c r="B27" t="s">
-        <v>199</v>
+        <v>220</v>
       </c>
       <c r="C27" t="s">
         <v>125</v>
@@ -1894,6 +1917,9 @@
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B28" t="s">
+        <v>220</v>
+      </c>
       <c r="C28" t="s">
         <v>128</v>
       </c>
@@ -1917,6 +1943,9 @@
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B29" t="s">
+        <v>220</v>
+      </c>
       <c r="C29" t="s">
         <v>131</v>
       </c>
@@ -1940,6 +1969,9 @@
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B30" t="s">
+        <v>220</v>
+      </c>
       <c r="C30" t="s">
         <v>134</v>
       </c>
@@ -1963,6 +1995,9 @@
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B31" t="s">
+        <v>220</v>
+      </c>
       <c r="C31" t="s">
         <v>137</v>
       </c>
@@ -2073,6 +2108,9 @@
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B35" t="s">
+        <v>220</v>
+      </c>
       <c r="C35" t="s">
         <v>153</v>
       </c>
@@ -2096,6 +2134,9 @@
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B36" t="s">
+        <v>220</v>
+      </c>
       <c r="C36" t="s">
         <v>159</v>
       </c>
@@ -2119,6 +2160,9 @@
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B37" t="s">
+        <v>220</v>
+      </c>
       <c r="C37" t="s">
         <v>162</v>
       </c>
@@ -2142,11 +2186,8 @@
       </c>
     </row>
     <row r="38" spans="1:9" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A38" t="s">
-        <v>211</v>
-      </c>
       <c r="B38" t="s">
-        <v>204</v>
+        <v>220</v>
       </c>
       <c r="C38" t="s">
         <v>165</v>
@@ -2171,11 +2212,8 @@
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A39" t="s">
-        <v>211</v>
-      </c>
       <c r="B39" t="s">
-        <v>204</v>
+        <v>220</v>
       </c>
       <c r="C39" t="s">
         <v>168</v>
@@ -2200,11 +2238,8 @@
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A40" t="s">
-        <v>211</v>
-      </c>
       <c r="B40" t="s">
-        <v>204</v>
+        <v>220</v>
       </c>
       <c r="C40" t="s">
         <v>173</v>
@@ -2229,6 +2264,9 @@
       </c>
     </row>
     <row r="41" spans="1:9" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="B41" t="s">
+        <v>220</v>
+      </c>
       <c r="C41" t="s">
         <v>176</v>
       </c>
@@ -2252,6 +2290,9 @@
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B42" t="s">
+        <v>220</v>
+      </c>
       <c r="C42" t="s">
         <v>179</v>
       </c>
@@ -2275,6 +2316,12 @@
       </c>
     </row>
     <row r="43" spans="1:9" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>216</v>
+      </c>
+      <c r="B43" t="s">
+        <v>220</v>
+      </c>
       <c r="C43" t="s">
         <v>185</v>
       </c>
@@ -2302,7 +2349,7 @@
         <v>209</v>
       </c>
       <c r="B44" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="C44" t="s">
         <v>189</v>
@@ -2333,7 +2380,7 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
         <x14:dataValidation type="list" operator="equal" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{2BD639CC-7032-4DDA-83A6-90D67489068F}">
           <x14:formula1>
-            <xm:f>Homologadores!$A$19:$A$27</xm:f>
+            <xm:f>Homologadores!$A$19:$A$28</xm:f>
           </x14:formula1>
           <xm:sqref>B2:B44</xm:sqref>
         </x14:dataValidation>
@@ -2351,7 +2398,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{659D4760-CAB5-44F6-8F8E-F56F7A47BDF9}">
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36.109375" bestFit="1" customWidth="1"/>
@@ -2465,26 +2512,31 @@
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>200</v>
+        <v>220</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
         <v>208</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dados da homologacao - 21/07/2026  9:17
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6565F183-9816-4344-97B9-3416FEF10E54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE61926B-2993-4180-B8C0-A1C085E4970E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="222">
   <si>
     <t>PENDENTE</t>
   </si>
@@ -719,6 +719,9 @@
   </si>
   <si>
     <t>Aguadando cenários</t>
+  </si>
+  <si>
+    <t>Aguardando Correção  (Avaliado)</t>
   </si>
 </sst>
 </file>
@@ -1181,32 +1184,32 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="72" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+    <row r="2" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="10" t="s">
         <v>216</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="C2" s="4" t="s">
+      <c r="B2" s="10" t="s">
+        <v>201</v>
+      </c>
+      <c r="C2" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="11" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1268,7 +1271,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>216</v>
       </c>
@@ -1356,35 +1359,35 @@
       </c>
     </row>
     <row r="8" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
-        <v>216</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="C8" s="4" t="s">
+      <c r="A8" s="10" t="s">
+        <v>212</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>201</v>
+      </c>
+      <c r="C8" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="G8" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="H8" s="4" t="s">
+      <c r="H8" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="I8" s="5" t="s">
+      <c r="I8" s="11" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
         <v>209</v>
       </c>
@@ -1413,7 +1416,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
         <v>212</v>
       </c>
@@ -1442,7 +1445,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="8" t="s">
         <v>209</v>
       </c>
@@ -1471,12 +1474,12 @@
         <v>61</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="172.8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A12" s="8" t="s">
         <v>209</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>201</v>
+        <v>221</v>
       </c>
       <c r="C12" s="8" t="s">
         <v>62</v>
@@ -1501,31 +1504,31 @@
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A13" s="4" t="s">
-        <v>214</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="C13" s="4" t="s">
+      <c r="A13" s="10" t="s">
+        <v>216</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>201</v>
+      </c>
+      <c r="C13" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="F13" s="4" t="s">
+      <c r="F13" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="G13" s="4" t="s">
+      <c r="G13" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="H13" s="4" t="s">
+      <c r="H13" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="I13" s="4" t="s">
+      <c r="I13" s="10" t="s">
         <v>72</v>
       </c>
     </row>
@@ -1559,35 +1562,35 @@
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="10" t="s">
         <v>212</v>
       </c>
-      <c r="B15" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="C15" s="4" t="s">
+      <c r="B15" s="10" t="s">
+        <v>201</v>
+      </c>
+      <c r="C15" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D15" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="E15" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="F15" s="4" t="s">
+      <c r="F15" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="G15" s="4" t="s">
+      <c r="G15" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="H15" s="4" t="s">
+      <c r="H15" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="I15" s="4" t="s">
+      <c r="I15" s="10" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="10" t="s">
         <v>214</v>
       </c>
@@ -1732,7 +1735,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>216</v>
       </c>
@@ -1761,7 +1764,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" s="8" t="s">
         <v>216</v>
       </c>
@@ -1877,12 +1880,12 @@
         <v>121</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A26" s="8" t="s">
         <v>216</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>217</v>
+        <v>201</v>
       </c>
       <c r="C26" s="8" t="s">
         <v>122</v>
@@ -1910,7 +1913,9 @@
       <c r="A27" s="8" t="s">
         <v>216</v>
       </c>
-      <c r="B27" s="8"/>
+      <c r="B27" s="8" t="s">
+        <v>200</v>
+      </c>
       <c r="C27" s="8" t="s">
         <v>125</v>
       </c>
@@ -1934,8 +1939,12 @@
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A28" s="8"/>
-      <c r="B28" s="8"/>
+      <c r="A28" s="8" t="s">
+        <v>216</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>200</v>
+      </c>
       <c r="C28" s="8" t="s">
         <v>128</v>
       </c>
@@ -1986,8 +1995,12 @@
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A30" s="8"/>
-      <c r="B30" s="8"/>
+      <c r="A30" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>201</v>
+      </c>
       <c r="C30" s="8" t="s">
         <v>134</v>
       </c>
@@ -2011,8 +2024,12 @@
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A31" s="8"/>
-      <c r="B31" s="8"/>
+      <c r="A31" s="8" t="s">
+        <v>216</v>
+      </c>
+      <c r="B31" s="8" t="s">
+        <v>200</v>
+      </c>
       <c r="C31" s="8" t="s">
         <v>137</v>
       </c>
@@ -2203,7 +2220,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="38" spans="1:9" ht="172.8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:9" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A38" s="8"/>
       <c r="B38" s="8" t="s">
         <v>220</v>
@@ -2284,7 +2301,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="41" spans="1:9" ht="201.6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:9" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A41" s="8"/>
       <c r="B41" s="8" t="s">
         <v>220</v>
@@ -2338,7 +2355,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="230.4" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:9" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A43" s="8" t="s">
         <v>216</v>
       </c>
@@ -2372,7 +2389,7 @@
         <v>209</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>201</v>
+        <v>221</v>
       </c>
       <c r="C44" s="8" t="s">
         <v>189</v>
@@ -2403,7 +2420,7 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
         <x14:dataValidation type="list" operator="equal" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{2BD639CC-7032-4DDA-83A6-90D67489068F}">
           <x14:formula1>
-            <xm:f>Homologadores!$A$19:$A$28</xm:f>
+            <xm:f>Homologadores!$A$19:$A$29</xm:f>
           </x14:formula1>
           <xm:sqref>B2:B44</xm:sqref>
         </x14:dataValidation>
@@ -2421,7 +2438,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{659D4760-CAB5-44F6-8F8E-F56F7A47BDF9}">
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36.109375" bestFit="1" customWidth="1"/>
@@ -2535,31 +2552,36 @@
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>200</v>
+        <v>220</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
         <v>208</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dados da homologacao - 21/07/2026 17:13
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,14 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE61926B-2993-4180-B8C0-A1C085E4970E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A112622B-C4CD-472A-A0FD-7ED6C9E1ACA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cenários homologação" sheetId="6" r:id="rId1"/>
     <sheet name="Homologadores" sheetId="8" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cenários homologação'!$B$1:$B$44</definedName>
+  </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -40,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="222">
   <si>
     <t>PENDENTE</t>
   </si>
@@ -676,9 +679,6 @@
     <t>08563524623</t>
   </si>
   <si>
-    <t xml:space="preserve">Aguardando </t>
-  </si>
-  <si>
     <t>51548569534</t>
   </si>
   <si>
@@ -722,6 +722,9 @@
   </si>
   <si>
     <t>Aguardando Correção  (Avaliado)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Em Correção </t>
   </si>
 </sst>
 </file>
@@ -745,7 +748,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -761,18 +764,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2" tint="-9.9978637043366805E-2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -804,29 +795,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1141,7 +1121,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C39B64EC-B305-411B-89CD-90AE48303B1A}">
-  <dimension ref="A1:I44"/>
+  <dimension ref="A1:K44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.5546875" bestFit="1" customWidth="1"/>
@@ -1155,7 +1135,7 @@
     <col min="9" max="9" width="111.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>1</v>
       </c>
@@ -1184,38 +1164,40 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="10" t="s">
+    <row r="2" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>216</v>
       </c>
-      <c r="B2" s="10" t="s">
-        <v>201</v>
-      </c>
-      <c r="C2" s="10" t="s">
+      <c r="C2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="D2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="10" t="s">
+      <c r="E2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="10" t="s">
+      <c r="F2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="G2" s="10" t="s">
+      <c r="G2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="10" t="s">
+      <c r="H2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="I2" s="11" t="s">
+      <c r="I2" s="5" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J2" s="6"/>
+      <c r="K2" s="6"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>200</v>
@@ -1241,13 +1223,15 @@
       <c r="I3" s="4" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J3" s="6"/>
+      <c r="K3" s="6"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>23</v>
@@ -1270,13 +1254,15 @@
       <c r="I4" s="4" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="J4" s="6"/>
+      <c r="K4" s="6"/>
+    </row>
+    <row r="5" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>28</v>
@@ -1299,10 +1285,12 @@
       <c r="I5" s="5" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J5" s="6"/>
+      <c r="K5" s="6"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>200</v>
@@ -1328,303 +1316,325 @@
       <c r="I6" s="4" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" s="6" t="s">
+      <c r="J6" s="6"/>
+      <c r="K6" s="6"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+    </row>
+    <row r="8" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
         <v>211</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B8" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="J8" s="6"/>
+      <c r="K8" s="6"/>
+    </row>
+    <row r="9" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A9" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J9" s="6"/>
+      <c r="K9" s="6"/>
+    </row>
+    <row r="10" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="J10" s="6"/>
+      <c r="K10" s="6"/>
+    </row>
+    <row r="11" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="I11" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="J11" s="6"/>
+      <c r="K11" s="6"/>
+    </row>
+    <row r="12" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A12" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="I12" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="J12" s="6"/>
+      <c r="K12" s="6"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A13" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="J13" s="6"/>
+      <c r="K13" s="6"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A14" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>204</v>
       </c>
-      <c r="C7" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="D7" s="7" t="s">
+      <c r="C14" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="J14" s="6"/>
+      <c r="K14" s="6"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A15" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I15" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="J15" s="6"/>
+      <c r="K15" s="6"/>
+    </row>
+    <row r="16" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A16" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I16" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="J16" s="6"/>
+      <c r="K16" s="6"/>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A17" s="4" t="s">
         <v>215</v>
       </c>
-      <c r="E7" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="G7" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="I7" s="6" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A8" s="10" t="s">
-        <v>212</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>201</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="D8" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="F8" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="G8" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="H8" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="I8" s="11" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A9" s="8" t="s">
-        <v>209</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>201</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="E9" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="G9" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="H9" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="I9" s="9" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A10" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>201</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="E10" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="F10" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="G10" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="H10" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="I10" s="9" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="8" t="s">
-        <v>209</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>201</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="D11" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="E11" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="F11" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="G11" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="H11" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="I11" s="9" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A12" s="8" t="s">
-        <v>209</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>221</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="D12" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="E12" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="F12" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="G12" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="H12" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="I12" s="9" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A13" s="10" t="s">
-        <v>216</v>
-      </c>
-      <c r="B13" s="10" t="s">
-        <v>201</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="D13" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="E13" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="F13" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="G13" s="10" t="s">
-        <v>70</v>
-      </c>
-      <c r="H13" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="I13" s="10" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A14" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="D14" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="E14" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="F14" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G14" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="H14" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="I14" s="6" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A15" s="10" t="s">
-        <v>212</v>
-      </c>
-      <c r="B15" s="10" t="s">
-        <v>201</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="D15" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="E15" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="F15" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="G15" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="H15" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="I15" s="10" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A16" s="10" t="s">
-        <v>214</v>
-      </c>
-      <c r="B16" s="10" t="s">
-        <v>201</v>
-      </c>
-      <c r="C16" s="10" t="s">
-        <v>82</v>
-      </c>
-      <c r="D16" s="10" t="s">
-        <v>83</v>
-      </c>
-      <c r="E16" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="F16" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="G16" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="H16" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="I16" s="11" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A17" s="4" t="s">
-        <v>216</v>
-      </c>
       <c r="B17" s="4" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>85</v>
@@ -1647,97 +1657,105 @@
       <c r="I17" s="4" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A18" s="8" t="s">
-        <v>216</v>
-      </c>
-      <c r="B18" s="8" t="s">
+      <c r="J17" s="6"/>
+      <c r="K17" s="6"/>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B18" s="4" t="s">
         <v>201</v>
       </c>
-      <c r="C18" s="8" t="s">
+      <c r="C18" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="D18" s="8" t="s">
+      <c r="D18" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="E18" s="8" t="s">
+      <c r="E18" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="F18" s="10" t="s">
+      <c r="F18" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="G18" s="8" t="s">
+      <c r="G18" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="H18" s="8" t="s">
+      <c r="H18" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="I18" s="8" t="s">
+      <c r="I18" s="4" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A19" s="8" t="s">
-        <v>216</v>
-      </c>
-      <c r="B19" s="8" t="s">
-        <v>217</v>
-      </c>
-      <c r="C19" s="8" t="s">
+      <c r="J18" s="6"/>
+      <c r="K18" s="6"/>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A19" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="C19" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="D19" s="8" t="s">
+      <c r="D19" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="E19" s="8" t="s">
+      <c r="E19" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="F19" s="10" t="s">
+      <c r="F19" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="G19" s="8" t="s">
+      <c r="G19" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="H19" s="8" t="s">
+      <c r="H19" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="I19" s="8" t="s">
+      <c r="I19" s="4" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A20" s="8" t="s">
-        <v>216</v>
-      </c>
-      <c r="B20" s="8" t="s">
-        <v>201</v>
-      </c>
-      <c r="C20" s="8" t="s">
+      <c r="J19" s="6"/>
+      <c r="K19" s="6"/>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A20" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C20" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="D20" s="8" t="s">
+      <c r="D20" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="E20" s="8" t="s">
+      <c r="E20" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="F20" s="10" t="s">
+      <c r="F20" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="G20" s="8" t="s">
+      <c r="G20" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="H20" s="8" t="s">
+      <c r="H20" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="I20" s="8" t="s">
+      <c r="I20" s="4" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="21" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="J20" s="6"/>
+      <c r="K20" s="6"/>
+    </row>
+    <row r="21" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B21" s="4" t="s">
         <v>200</v>
@@ -1763,39 +1781,43 @@
       <c r="I21" s="5" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="22" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A22" s="8" t="s">
-        <v>216</v>
-      </c>
-      <c r="B22" s="8" t="s">
+      <c r="J21" s="6"/>
+      <c r="K21" s="6"/>
+    </row>
+    <row r="22" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A22" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B22" s="4" t="s">
         <v>201</v>
       </c>
-      <c r="C22" s="8" t="s">
+      <c r="C22" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="D22" s="8" t="s">
+      <c r="D22" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="E22" s="8" t="s">
+      <c r="E22" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="F22" s="8" t="s">
+      <c r="F22" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="G22" s="8" t="s">
+      <c r="G22" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="H22" s="8" t="s">
+      <c r="H22" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="I22" s="9" t="s">
+      <c r="I22" s="5" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J22" s="6"/>
+      <c r="K22" s="6"/>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>200</v>
@@ -1821,599 +1843,648 @@
       <c r="I23" s="4" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A24" s="8" t="s">
+      <c r="J23" s="6"/>
+      <c r="K23" s="6"/>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A24" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="H24" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="I24" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="J24" s="6"/>
+      <c r="K24" s="6"/>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A25" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="H25" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="I25" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="J25" s="6"/>
+      <c r="K25" s="6"/>
+    </row>
+    <row r="26" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A26" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="H26" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="I26" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="J26" s="6"/>
+      <c r="K26" s="6"/>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A27" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="I27" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="J27" s="6"/>
+      <c r="K27" s="6"/>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A28" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="G28" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="H28" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="I28" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="J28" s="6"/>
+      <c r="K28" s="6"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A29" s="4"/>
+      <c r="B29" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G29" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="H29" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="I29" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="J29" s="6"/>
+      <c r="K29" s="6"/>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A30" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="G30" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="H30" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="I30" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="J30" s="6"/>
+      <c r="K30" s="6"/>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A31" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="G31" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="H31" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="I31" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="J31" s="6"/>
+      <c r="K31" s="6"/>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A32" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="G32" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="H32" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="I32" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="J32" s="6"/>
+      <c r="K32" s="6"/>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A33" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="G33" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="H33" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="I33" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="J33" s="6"/>
+      <c r="K33" s="6"/>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A34" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="G34" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="H34" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="I34" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="J34" s="6"/>
+      <c r="K34" s="6"/>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A35" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G35" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="H35" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="I35" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="J35" s="6"/>
+      <c r="K35" s="6"/>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A36" s="4"/>
+      <c r="B36" s="4" t="s">
         <v>216</v>
       </c>
-      <c r="B24" s="8" t="s">
+      <c r="C36" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="F36" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="G36" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="H36" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="I36" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="J36" s="6"/>
+      <c r="K36" s="6"/>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A37" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="D37" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="E37" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="F37" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G37" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="H37" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="I37" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="J37" s="6"/>
+      <c r="K37" s="6"/>
+    </row>
+    <row r="38" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A38" s="4"/>
+      <c r="B38" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="D38" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="E38" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="F38" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G38" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="H38" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="I38" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="J38" s="6"/>
+      <c r="K38" s="6"/>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A39" s="4"/>
+      <c r="B39" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G39" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="H39" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="I39" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="J39" s="6"/>
+      <c r="K39" s="6"/>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A40" s="4"/>
+      <c r="B40" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="F40" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G40" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="H40" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="I40" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="J40" s="6"/>
+      <c r="K40" s="6"/>
+    </row>
+    <row r="41" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A41" s="4"/>
+      <c r="B41" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="D41" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G41" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="H41" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="I41" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="J41" s="6"/>
+      <c r="K41" s="6"/>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A42" s="4"/>
+      <c r="B42" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="D42" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="E42" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="F42" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="G42" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="H42" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="I42" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="J42" s="6"/>
+      <c r="K42" s="6"/>
+    </row>
+    <row r="43" spans="1:11" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A43" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="D43" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="E43" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="F43" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="G43" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="H43" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="I43" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="J43" s="6"/>
+      <c r="K43" s="6"/>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A44" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="B44" s="4" t="s">
         <v>201</v>
       </c>
-      <c r="C24" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="D24" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="E24" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="F24" s="8" t="s">
+      <c r="C44" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="D44" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="E44" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="F44" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="G24" s="8" t="s">
+      <c r="G44" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="H24" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="I24" s="8" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A25" s="8" t="s">
-        <v>216</v>
-      </c>
-      <c r="B25" s="8" t="s">
-        <v>217</v>
-      </c>
-      <c r="C25" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="D25" s="8" t="s">
-        <v>117</v>
-      </c>
-      <c r="E25" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="F25" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="G25" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="H25" s="8" t="s">
-        <v>120</v>
-      </c>
-      <c r="I25" s="8" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A26" s="8" t="s">
-        <v>216</v>
-      </c>
-      <c r="B26" s="8" t="s">
-        <v>201</v>
-      </c>
-      <c r="C26" s="8" t="s">
-        <v>122</v>
-      </c>
-      <c r="D26" s="8" t="s">
-        <v>123</v>
-      </c>
-      <c r="E26" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="F26" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="G26" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="H26" s="8" t="s">
-        <v>120</v>
-      </c>
-      <c r="I26" s="9" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A27" s="8" t="s">
-        <v>216</v>
-      </c>
-      <c r="B27" s="8" t="s">
-        <v>200</v>
-      </c>
-      <c r="C27" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="D27" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="E27" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="F27" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="G27" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="H27" s="8" t="s">
-        <v>120</v>
-      </c>
-      <c r="I27" s="8" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A28" s="8" t="s">
-        <v>216</v>
-      </c>
-      <c r="B28" s="8" t="s">
-        <v>200</v>
-      </c>
-      <c r="C28" s="8" t="s">
-        <v>128</v>
-      </c>
-      <c r="D28" s="8" t="s">
-        <v>129</v>
-      </c>
-      <c r="E28" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="F28" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="G28" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="H28" s="8" t="s">
-        <v>120</v>
-      </c>
-      <c r="I28" s="8" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A29" s="8"/>
-      <c r="B29" s="8" t="s">
-        <v>220</v>
-      </c>
-      <c r="C29" s="8" t="s">
-        <v>131</v>
-      </c>
-      <c r="D29" s="8" t="s">
-        <v>132</v>
-      </c>
-      <c r="E29" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="F29" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="G29" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="H29" s="8" t="s">
-        <v>120</v>
-      </c>
-      <c r="I29" s="8" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A30" s="8" t="s">
-        <v>214</v>
-      </c>
-      <c r="B30" s="8" t="s">
-        <v>201</v>
-      </c>
-      <c r="C30" s="8" t="s">
-        <v>134</v>
-      </c>
-      <c r="D30" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="E30" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="F30" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="G30" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="H30" s="8" t="s">
-        <v>120</v>
-      </c>
-      <c r="I30" s="8" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A31" s="8" t="s">
-        <v>216</v>
-      </c>
-      <c r="B31" s="8" t="s">
-        <v>200</v>
-      </c>
-      <c r="C31" s="8" t="s">
-        <v>137</v>
-      </c>
-      <c r="D31" s="8" t="s">
-        <v>138</v>
-      </c>
-      <c r="E31" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="F31" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="G31" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="H31" s="8" t="s">
-        <v>120</v>
-      </c>
-      <c r="I31" s="8" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A32" s="8" t="s">
-        <v>211</v>
-      </c>
-      <c r="B32" s="8" t="s">
-        <v>204</v>
-      </c>
-      <c r="C32" s="8" t="s">
-        <v>140</v>
-      </c>
-      <c r="D32" s="8" t="s">
-        <v>141</v>
-      </c>
-      <c r="E32" s="8" t="s">
-        <v>142</v>
-      </c>
-      <c r="F32" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="G32" s="8" t="s">
-        <v>143</v>
-      </c>
-      <c r="H32" s="8" t="s">
-        <v>144</v>
-      </c>
-      <c r="I32" s="8" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A33" s="8" t="s">
-        <v>211</v>
-      </c>
-      <c r="B33" s="8" t="s">
-        <v>204</v>
-      </c>
-      <c r="C33" s="8" t="s">
-        <v>146</v>
-      </c>
-      <c r="D33" s="8" t="s">
-        <v>147</v>
-      </c>
-      <c r="E33" s="8" t="s">
-        <v>142</v>
-      </c>
-      <c r="F33" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="G33" s="8" t="s">
-        <v>143</v>
-      </c>
-      <c r="H33" s="8" t="s">
-        <v>144</v>
-      </c>
-      <c r="I33" s="8" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A34" s="8" t="s">
-        <v>211</v>
-      </c>
-      <c r="B34" s="8" t="s">
-        <v>204</v>
-      </c>
-      <c r="C34" s="8" t="s">
-        <v>149</v>
-      </c>
-      <c r="D34" s="8" t="s">
-        <v>150</v>
-      </c>
-      <c r="E34" s="8" t="s">
-        <v>142</v>
-      </c>
-      <c r="F34" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="G34" s="8" t="s">
-        <v>151</v>
-      </c>
-      <c r="H34" s="8" t="s">
-        <v>144</v>
-      </c>
-      <c r="I34" s="8" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A35" s="8"/>
-      <c r="B35" s="8" t="s">
-        <v>220</v>
-      </c>
-      <c r="C35" s="8" t="s">
-        <v>153</v>
-      </c>
-      <c r="D35" s="8" t="s">
-        <v>154</v>
-      </c>
-      <c r="E35" s="8" t="s">
-        <v>155</v>
-      </c>
-      <c r="F35" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="G35" s="8" t="s">
-        <v>156</v>
-      </c>
-      <c r="H35" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="I35" s="8" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A36" s="8"/>
-      <c r="B36" s="8" t="s">
-        <v>220</v>
-      </c>
-      <c r="C36" s="8" t="s">
-        <v>159</v>
-      </c>
-      <c r="D36" s="8" t="s">
-        <v>160</v>
-      </c>
-      <c r="E36" s="8" t="s">
-        <v>155</v>
-      </c>
-      <c r="F36" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="G36" s="8" t="s">
-        <v>156</v>
-      </c>
-      <c r="H36" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="I36" s="8" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A37" s="8"/>
-      <c r="B37" s="8" t="s">
-        <v>220</v>
-      </c>
-      <c r="C37" s="8" t="s">
-        <v>162</v>
-      </c>
-      <c r="D37" s="8" t="s">
-        <v>163</v>
-      </c>
-      <c r="E37" s="8" t="s">
-        <v>155</v>
-      </c>
-      <c r="F37" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="G37" s="8" t="s">
-        <v>156</v>
-      </c>
-      <c r="H37" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="I37" s="8" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A38" s="8"/>
-      <c r="B38" s="8" t="s">
-        <v>220</v>
-      </c>
-      <c r="C38" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="D38" s="9" t="s">
-        <v>166</v>
-      </c>
-      <c r="E38" s="8" t="s">
-        <v>155</v>
-      </c>
-      <c r="F38" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="G38" s="8" t="s">
-        <v>156</v>
-      </c>
-      <c r="H38" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="I38" s="8" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A39" s="8"/>
-      <c r="B39" s="8" t="s">
-        <v>220</v>
-      </c>
-      <c r="C39" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="D39" s="8" t="s">
-        <v>169</v>
-      </c>
-      <c r="E39" s="8" t="s">
-        <v>170</v>
-      </c>
-      <c r="F39" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="G39" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="H39" s="8" t="s">
-        <v>171</v>
-      </c>
-      <c r="I39" s="8" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A40" s="8"/>
-      <c r="B40" s="8" t="s">
-        <v>220</v>
-      </c>
-      <c r="C40" s="8" t="s">
-        <v>173</v>
-      </c>
-      <c r="D40" s="8" t="s">
-        <v>174</v>
-      </c>
-      <c r="E40" s="8" t="s">
-        <v>170</v>
-      </c>
-      <c r="F40" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="G40" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="H40" s="8" t="s">
-        <v>171</v>
-      </c>
-      <c r="I40" s="8" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A41" s="8"/>
-      <c r="B41" s="8" t="s">
-        <v>220</v>
-      </c>
-      <c r="C41" s="8" t="s">
-        <v>176</v>
-      </c>
-      <c r="D41" s="9" t="s">
-        <v>177</v>
-      </c>
-      <c r="E41" s="8" t="s">
-        <v>170</v>
-      </c>
-      <c r="F41" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="G41" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="H41" s="8" t="s">
-        <v>171</v>
-      </c>
-      <c r="I41" s="8" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A42" s="8"/>
-      <c r="B42" s="8" t="s">
-        <v>220</v>
-      </c>
-      <c r="C42" s="8" t="s">
-        <v>179</v>
-      </c>
-      <c r="D42" s="8" t="s">
-        <v>180</v>
-      </c>
-      <c r="E42" s="8" t="s">
-        <v>181</v>
-      </c>
-      <c r="F42" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="G42" s="8" t="s">
-        <v>182</v>
-      </c>
-      <c r="H42" s="8" t="s">
+      <c r="H44" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="I42" s="8" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A43" s="8" t="s">
-        <v>216</v>
-      </c>
-      <c r="B43" s="8" t="s">
-        <v>220</v>
-      </c>
-      <c r="C43" s="8" t="s">
-        <v>185</v>
-      </c>
-      <c r="D43" s="9" t="s">
-        <v>186</v>
-      </c>
-      <c r="E43" s="8" t="s">
-        <v>181</v>
-      </c>
-      <c r="F43" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="G43" s="8" t="s">
-        <v>187</v>
-      </c>
-      <c r="H43" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="I43" s="8" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A44" s="8" t="s">
-        <v>209</v>
-      </c>
-      <c r="B44" s="8" t="s">
-        <v>221</v>
-      </c>
-      <c r="C44" s="8" t="s">
-        <v>189</v>
-      </c>
-      <c r="D44" s="8" t="s">
-        <v>190</v>
-      </c>
-      <c r="E44" s="8" t="s">
-        <v>181</v>
-      </c>
-      <c r="F44" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="G44" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="H44" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="I44" s="8" t="s">
+      <c r="I44" s="4" t="s">
         <v>191</v>
       </c>
+      <c r="J44" s="6"/>
+      <c r="K44" s="6"/>
     </row>
   </sheetData>
+  <autoFilter ref="B1:B44" xr:uid="{C39B64EC-B305-411B-89CD-90AE48303B1A}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -2466,12 +2537,12 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>197</v>
@@ -2482,24 +2553,24 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>202</v>
@@ -2510,7 +2581,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>205</v>
@@ -2521,10 +2592,10 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C9" t="s">
         <v>203</v>
@@ -2542,22 +2613,22 @@
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.3">
@@ -2577,12 +2648,12 @@
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>206</v>
+        <v>221</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza dados da homologacao - 21/07/2026 17:14
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A112622B-C4CD-472A-A0FD-7ED6C9E1ACA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B7012E8-34F4-49FE-859E-D391757388EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1126,7 +1126,7 @@
   <cols>
     <col min="1" max="1" width="15.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="27.88671875" customWidth="1"/>
-    <col min="3" max="3" width="9" customWidth="1"/>
+    <col min="3" max="3" width="18" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="103.109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="22.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="20.88671875" bestFit="1" customWidth="1"/>

</xml_diff>

<commit_message>
Evolucao agora le aba ResumoDiario da planilha, remove snapshots
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B7012E8-34F4-49FE-859E-D391757388EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C700A07E-83CA-440A-A0C5-7C1F132CE1B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cenários homologação" sheetId="6" r:id="rId1"/>
     <sheet name="Homologadores" sheetId="8" r:id="rId2"/>
+    <sheet name="ResumoDiario" sheetId="9" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cenários homologação'!$B$1:$B$44</definedName>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="230">
   <si>
     <t>PENDENTE</t>
   </si>
@@ -725,13 +726,37 @@
   </si>
   <si>
     <t xml:space="preserve">Em Correção </t>
+  </si>
+  <si>
+    <t>Pendente de cenário</t>
+  </si>
+  <si>
+    <t>Homologado com ressalva</t>
+  </si>
+  <si>
+    <t>Disponível para reteste</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Atual</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Em Correção</t>
+  </si>
+  <si>
+    <t>Em Análise</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -743,6 +768,13 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -795,7 +827,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -807,6 +839,19 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="22" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2659,4 +2704,154 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E94EB92-949A-4861-8A92-72A5C32EFB43}">
+  <dimension ref="A1:I6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="21.77734375" customWidth="1"/>
+    <col min="2" max="2" width="19" customWidth="1"/>
+    <col min="3" max="3" width="20.109375" customWidth="1"/>
+    <col min="4" max="4" width="18.88671875" customWidth="1"/>
+    <col min="5" max="5" width="28.88671875" customWidth="1"/>
+    <col min="6" max="6" width="30.6640625" customWidth="1"/>
+    <col min="7" max="7" width="22.21875" customWidth="1"/>
+    <col min="8" max="8" width="24.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A1" s="8"/>
+      <c r="B1" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>229</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>200</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>223</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>224</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2" s="10" t="s">
+        <v>226</v>
+      </c>
+      <c r="B2" s="10">
+        <v>8</v>
+      </c>
+      <c r="C2" s="10">
+        <v>2</v>
+      </c>
+      <c r="D2" s="10">
+        <v>1</v>
+      </c>
+      <c r="E2" s="10">
+        <v>8</v>
+      </c>
+      <c r="F2" s="10">
+        <v>4</v>
+      </c>
+      <c r="G2" s="10">
+        <v>2</v>
+      </c>
+      <c r="H2" s="10">
+        <v>13</v>
+      </c>
+      <c r="I2" s="7">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" s="11">
+        <v>46224.375</v>
+      </c>
+      <c r="B3" s="10">
+        <v>11</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>227</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>227</v>
+      </c>
+      <c r="E3" s="10">
+        <v>6</v>
+      </c>
+      <c r="F3" s="10">
+        <v>4</v>
+      </c>
+      <c r="G3" s="10">
+        <v>1</v>
+      </c>
+      <c r="H3" s="10">
+        <v>16</v>
+      </c>
+      <c r="I3" s="7">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" s="11">
+        <v>46225.375</v>
+      </c>
+      <c r="B4" s="10"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="10"/>
+      <c r="H4" s="10"/>
+      <c r="I4" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" s="11">
+        <v>46226.375</v>
+      </c>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="10"/>
+      <c r="I5" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" s="11">
+        <v>46227.375</v>
+      </c>
+      <c r="B6" s="10"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
+      <c r="I6" s="7">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza dados da homologacao - 21/07/2026 17:37
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C700A07E-83CA-440A-A0C5-7C1F132CE1B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A952184-095F-4B6D-BA32-34690CD0F571}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cenários homologação" sheetId="6" r:id="rId1"/>
@@ -1245,7 +1245,7 @@
         <v>215</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>16</v>
@@ -1462,7 +1462,7 @@
         <v>211</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>201</v>
+        <v>221</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>53</v>

</xml_diff>

<commit_message>
Evolucao usa colunas Hora+Data da aba ResumoDiario, adiciona tabela de variacao entre dias
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A952184-095F-4B6D-BA32-34690CD0F571}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF2B5679-A6CA-4DF6-BE38-D1DA5F323EB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cenários homologação" sheetId="6" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="230">
   <si>
     <t>PENDENTE</t>
   </si>
@@ -740,23 +740,23 @@
     <t>Total</t>
   </si>
   <si>
-    <t>Atual</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
     <t>Em Correção</t>
   </si>
   <si>
     <t>Em Análise</t>
+  </si>
+  <si>
+    <t>Data</t>
+  </si>
+  <si>
+    <t>Hora</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -779,8 +779,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -796,6 +804,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -827,7 +841,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -839,19 +853,20 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="22" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2708,146 +2723,144 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E94EB92-949A-4861-8A92-72A5C32EFB43}">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.77734375" customWidth="1"/>
-    <col min="2" max="2" width="19" customWidth="1"/>
-    <col min="3" max="3" width="20.109375" customWidth="1"/>
-    <col min="4" max="4" width="18.88671875" customWidth="1"/>
-    <col min="5" max="5" width="28.88671875" customWidth="1"/>
-    <col min="6" max="6" width="30.6640625" customWidth="1"/>
-    <col min="7" max="7" width="22.21875" customWidth="1"/>
-    <col min="8" max="8" width="24.88671875" customWidth="1"/>
+    <col min="2" max="2" width="21.77734375" customWidth="1"/>
+    <col min="3" max="3" width="19" customWidth="1"/>
+    <col min="4" max="4" width="20.109375" customWidth="1"/>
+    <col min="5" max="5" width="18.88671875" customWidth="1"/>
+    <col min="6" max="6" width="28.88671875" customWidth="1"/>
+    <col min="7" max="7" width="30.6640625" customWidth="1"/>
+    <col min="8" max="8" width="22.21875" customWidth="1"/>
+    <col min="9" max="9" width="24.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="8"/>
-      <c r="B1" s="9" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>228</v>
+      </c>
+      <c r="C1" s="8" t="s">
         <v>222</v>
       </c>
-      <c r="C1" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="D1" s="9" t="s">
-        <v>229</v>
-      </c>
-      <c r="E1" s="9" t="s">
+      <c r="D1" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>227</v>
+      </c>
+      <c r="F1" s="8" t="s">
         <v>200</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="G1" s="8" t="s">
         <v>223</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="H1" s="8" t="s">
         <v>224</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="I1" s="8" t="s">
         <v>201</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="J1" s="8" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="10" t="s">
-        <v>226</v>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" s="9">
+        <v>0.70833333333333337</v>
       </c>
       <c r="B2" s="10">
+        <v>46224</v>
+      </c>
+      <c r="C2" s="11">
         <v>8</v>
       </c>
-      <c r="C2" s="10">
+      <c r="D2" s="11">
         <v>2</v>
       </c>
-      <c r="D2" s="10">
+      <c r="E2" s="11">
         <v>1</v>
       </c>
-      <c r="E2" s="10">
+      <c r="F2" s="11">
         <v>8</v>
       </c>
-      <c r="F2" s="10">
+      <c r="G2" s="11">
         <v>4</v>
       </c>
-      <c r="G2" s="10">
+      <c r="H2" s="11">
         <v>2</v>
       </c>
-      <c r="H2" s="10">
+      <c r="I2" s="11">
         <v>13</v>
       </c>
-      <c r="I2" s="7">
+      <c r="J2" s="12">
+        <f>C2+D2+E2+F2+G2+H2+I2</f>
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" s="11">
-        <v>46224.375</v>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="9">
+        <v>0.75</v>
       </c>
       <c r="B3" s="10">
+        <v>46225.375</v>
+      </c>
+      <c r="C3" s="11">
+        <v>6</v>
+      </c>
+      <c r="D3" s="11">
+        <v>0</v>
+      </c>
+      <c r="E3" s="11">
+        <v>3</v>
+      </c>
+      <c r="F3" s="11">
+        <v>10</v>
+      </c>
+      <c r="G3" s="11">
+        <v>5</v>
+      </c>
+      <c r="H3" s="11">
+        <v>3</v>
+      </c>
+      <c r="I3" s="11">
         <v>11</v>
       </c>
-      <c r="C3" s="10" t="s">
-        <v>227</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>227</v>
-      </c>
-      <c r="E3" s="10">
-        <v>6</v>
-      </c>
-      <c r="F3" s="10">
-        <v>4</v>
-      </c>
-      <c r="G3" s="10">
-        <v>1</v>
-      </c>
-      <c r="H3" s="10">
-        <v>16</v>
-      </c>
-      <c r="I3" s="7">
+      <c r="J3" s="12">
+        <f>C3+D3+E3+F3+G3+H3+I3</f>
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="11">
-        <v>46225.375</v>
-      </c>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" s="9"/>
       <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
-      <c r="H4" s="10"/>
-      <c r="I4" s="7">
+      <c r="C4" s="11"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="11"/>
+      <c r="F4" s="11"/>
+      <c r="G4" s="11"/>
+      <c r="H4" s="11"/>
+      <c r="I4" s="11"/>
+      <c r="J4" s="12">
+        <f t="shared" ref="J3:J5" si="0">C4+D4+E4+F4+G4+H4+I4</f>
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" s="11">
-        <v>46226.375</v>
-      </c>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" s="9"/>
       <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
-      <c r="G5" s="10"/>
-      <c r="H5" s="10"/>
-      <c r="I5" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" s="11">
-        <v>46227.375</v>
-      </c>
-      <c r="B6" s="10"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
-      <c r="F6" s="10"/>
-      <c r="G6" s="10"/>
-      <c r="H6" s="10"/>
-      <c r="I6" s="7">
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="11"/>
+      <c r="H5" s="11"/>
+      <c r="I5" s="11"/>
+      <c r="J5" s="12">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dados da homologacao - 22/07/2026 17:11
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF2B5679-A6CA-4DF6-BE38-D1DA5F323EB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B19A1AF7-7F9D-4821-B464-1400A8400978}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cenários homologação" sheetId="6" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="230">
   <si>
     <t>PENDENTE</t>
   </si>
@@ -1229,7 +1229,7 @@
         <v>215</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>216</v>
+        <v>207</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>10</v>
@@ -1415,7 +1415,7 @@
         <v>211</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>201</v>
+        <v>216</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>43</v>
@@ -1508,7 +1508,7 @@
         <v>208</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>221</v>
+        <v>201</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>59</v>
@@ -1539,7 +1539,7 @@
         <v>208</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>201</v>
+        <v>216</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>62</v>
@@ -1725,7 +1725,7 @@
         <v>215</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>201</v>
+        <v>221</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>88</v>
@@ -1911,7 +1911,7 @@
         <v>215</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>113</v>
@@ -1942,7 +1942,7 @@
         <v>215</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>201</v>
+        <v>221</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>116</v>
@@ -2277,9 +2277,11 @@
       <c r="K35" s="6"/>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A36" s="4"/>
+      <c r="A36" s="4" t="s">
+        <v>215</v>
+      </c>
       <c r="B36" s="4" t="s">
-        <v>216</v>
+        <v>200</v>
       </c>
       <c r="C36" s="4" t="s">
         <v>159</v>
@@ -2337,9 +2339,11 @@
       <c r="K37" s="6"/>
     </row>
     <row r="38" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A38" s="4"/>
+      <c r="A38" s="4" t="s">
+        <v>215</v>
+      </c>
       <c r="B38" s="4" t="s">
-        <v>219</v>
+        <v>200</v>
       </c>
       <c r="C38" s="4" t="s">
         <v>165</v>
@@ -2845,7 +2849,7 @@
       <c r="H4" s="11"/>
       <c r="I4" s="11"/>
       <c r="J4" s="12">
-        <f t="shared" ref="J3:J5" si="0">C4+D4+E4+F4+G4+H4+I4</f>
+        <f t="shared" ref="J4:J5" si="0">C4+D4+E4+F4+G4+H4+I4</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dados da homologacao - 22/07/2026 17:18
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B19A1AF7-7F9D-4821-B464-1400A8400978}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E21781B-4958-4855-A69E-7CF76AE2A95B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1446,7 +1446,7 @@
         <v>208</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>201</v>
+        <v>221</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>49</v>
@@ -2816,7 +2816,7 @@
         <v>6</v>
       </c>
       <c r="D3" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3" s="11">
         <v>3</v>
@@ -2831,7 +2831,7 @@
         <v>3</v>
       </c>
       <c r="I3" s="11">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J3" s="12">
         <f>C3+D3+E3+F3+G3+H3+I3</f>

</xml_diff>

<commit_message>
Atualiza dados da homologacao - 23/07/2026 15:35
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E21781B-4958-4855-A69E-7CF76AE2A95B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47261F98-85BB-43AF-9134-56C99DA5976C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -743,13 +743,13 @@
     <t>Em Correção</t>
   </si>
   <si>
-    <t>Em Análise</t>
-  </si>
-  <si>
     <t>Data</t>
   </si>
   <si>
     <t>Hora</t>
+  </si>
+  <si>
+    <t>Ag Correção</t>
   </si>
 </sst>
 </file>
@@ -1446,7 +1446,7 @@
         <v>208</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>49</v>
@@ -1570,7 +1570,7 @@
         <v>215</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>201</v>
+        <v>221</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>67</v>
@@ -1973,7 +1973,7 @@
         <v>215</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>122</v>
@@ -2459,7 +2459,7 @@
     <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A42" s="4"/>
       <c r="B42" s="4" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="C42" s="4" t="s">
         <v>179</v>
@@ -2490,7 +2490,7 @@
         <v>215</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="C43" s="4" t="s">
         <v>185</v>
@@ -2732,7 +2732,7 @@
   <cols>
     <col min="2" max="2" width="21.77734375" customWidth="1"/>
     <col min="3" max="3" width="19" customWidth="1"/>
-    <col min="4" max="4" width="20.109375" customWidth="1"/>
+    <col min="4" max="4" width="11.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18.88671875" customWidth="1"/>
     <col min="6" max="6" width="28.88671875" customWidth="1"/>
     <col min="7" max="7" width="30.6640625" customWidth="1"/>
@@ -2742,10 +2742,10 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C1" s="8" t="s">
         <v>222</v>
@@ -2754,7 +2754,7 @@
         <v>226</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="F1" s="8" t="s">
         <v>200</v>
@@ -2807,7 +2807,7 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="9">
-        <v>0.75</v>
+        <v>0.70833333333333337</v>
       </c>
       <c r="B3" s="10">
         <v>46225.375</v>
@@ -2839,18 +2839,36 @@
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" s="9"/>
-      <c r="B4" s="10"/>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="11"/>
-      <c r="G4" s="11"/>
-      <c r="H4" s="11"/>
-      <c r="I4" s="11"/>
+      <c r="A4" s="9">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="B4" s="10">
+        <v>46226</v>
+      </c>
+      <c r="C4" s="11">
+        <v>4</v>
+      </c>
+      <c r="D4" s="11">
+        <v>1</v>
+      </c>
+      <c r="E4" s="11">
+        <v>5</v>
+      </c>
+      <c r="F4" s="11">
+        <v>10</v>
+      </c>
+      <c r="G4" s="11">
+        <v>5</v>
+      </c>
+      <c r="H4" s="11">
+        <v>4</v>
+      </c>
+      <c r="I4" s="11">
+        <v>9</v>
+      </c>
       <c r="J4" s="12">
         <f t="shared" ref="J4:J5" si="0">C4+D4+E4+F4+G4+H4+I4</f>
-        <v>0</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Atualiza dados da homologacao - 23/07/2026 17:22
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47261F98-85BB-43AF-9134-56C99DA5976C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80F00638-374F-485A-A532-0D4E64BA46F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cenários homologação" sheetId="6" r:id="rId1"/>
@@ -1415,7 +1415,7 @@
         <v>211</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>216</v>
+        <v>201</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>43</v>
@@ -1446,7 +1446,7 @@
         <v>208</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>216</v>
+        <v>200</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>49</v>
@@ -1508,7 +1508,7 @@
         <v>208</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>201</v>
+        <v>216</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>59</v>
@@ -1539,7 +1539,7 @@
         <v>208</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>216</v>
+        <v>200</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>62</v>
@@ -1632,7 +1632,7 @@
         <v>211</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>77</v>
@@ -1849,7 +1849,7 @@
         <v>215</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>104</v>
@@ -1911,7 +1911,7 @@
         <v>215</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>216</v>
+        <v>200</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>113</v>
@@ -2095,7 +2095,7 @@
         <v>213</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>134</v>
@@ -2740,7 +2740,7 @@
     <col min="9" max="9" width="24.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
         <v>228</v>
       </c>
@@ -2855,16 +2855,16 @@
         <v>5</v>
       </c>
       <c r="F4" s="11">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G4" s="11">
+        <v>8</v>
+      </c>
+      <c r="H4" s="11">
+        <v>1</v>
+      </c>
+      <c r="I4" s="11">
         <v>5</v>
-      </c>
-      <c r="H4" s="11">
-        <v>4</v>
-      </c>
-      <c r="I4" s="11">
-        <v>9</v>
       </c>
       <c r="J4" s="12">
         <f t="shared" ref="J4:J5" si="0">C4+D4+E4+F4+G4+H4+I4</f>

</xml_diff>

<commit_message>
Atualiza dados da homologacao - 24/07/2026 15:38
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80F00638-374F-485A-A532-0D4E64BA46F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CBFA2A1-3B09-4450-A2AC-73BBCF1073A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1477,7 +1477,7 @@
         <v>211</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>221</v>
+        <v>200</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>53</v>
@@ -1508,7 +1508,7 @@
         <v>208</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>216</v>
+        <v>207</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>59</v>
@@ -1570,7 +1570,7 @@
         <v>215</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>221</v>
+        <v>207</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>67</v>
@@ -1663,7 +1663,7 @@
         <v>213</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>201</v>
+        <v>221</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>82</v>
@@ -1756,7 +1756,7 @@
         <v>215</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>201</v>
+        <v>221</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>91</v>
@@ -1942,7 +1942,7 @@
         <v>215</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>221</v>
+        <v>201</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>116</v>
@@ -2372,7 +2372,7 @@
     <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39" s="4"/>
       <c r="B39" s="4" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C39" s="4" t="s">
         <v>168</v>
@@ -2401,7 +2401,7 @@
     <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" s="4"/>
       <c r="B40" s="4" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="C40" s="4" t="s">
         <v>173</v>
@@ -2430,7 +2430,7 @@
     <row r="41" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A41" s="4"/>
       <c r="B41" s="4" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="C41" s="4" t="s">
         <v>176</v>
@@ -2872,18 +2872,36 @@
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" s="9"/>
-      <c r="B5" s="10"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
-      <c r="I5" s="11"/>
+      <c r="A5" s="9">
+        <v>0.64583333333333337</v>
+      </c>
+      <c r="B5" s="10">
+        <v>46227</v>
+      </c>
+      <c r="C5" s="11">
+        <v>1</v>
+      </c>
+      <c r="D5" s="11">
+        <v>1</v>
+      </c>
+      <c r="E5" s="11">
+        <v>6</v>
+      </c>
+      <c r="F5" s="11">
+        <v>15</v>
+      </c>
+      <c r="G5" s="11">
+        <v>10</v>
+      </c>
+      <c r="H5" s="11">
+        <v>1</v>
+      </c>
+      <c r="I5" s="11">
+        <v>4</v>
+      </c>
       <c r="J5" s="12">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza dados da homologacao - 24/07/2026 16:35
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CBFA2A1-3B09-4450-A2AC-73BBCF1073A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A0F8E8C-CFF2-4AE3-80B1-E1DEF9223B43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1415,7 +1415,7 @@
         <v>211</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>201</v>
+        <v>221</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>43</v>
@@ -1756,7 +1756,7 @@
         <v>215</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>221</v>
+        <v>201</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>91</v>
@@ -2372,7 +2372,7 @@
     <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39" s="4"/>
       <c r="B39" s="4" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="C39" s="4" t="s">
         <v>168</v>
@@ -2740,7 +2740,7 @@
     <col min="9" max="9" width="24.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
         <v>228</v>
       </c>
@@ -2885,7 +2885,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="11">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F5" s="11">
         <v>15</v>
@@ -2894,10 +2894,10 @@
         <v>10</v>
       </c>
       <c r="H5" s="11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I5" s="11">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J5" s="12">
         <f t="shared" si="0"/>

</xml_diff>

<commit_message>
Atualiza dados da homologacao - 24/07/2026 17:00
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A0F8E8C-CFF2-4AE3-80B1-E1DEF9223B43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E04B6AE-C57A-45A7-AB30-180A9E4FDBB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2521,7 +2521,7 @@
         <v>208</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C44" s="4" t="s">
         <v>189</v>
@@ -2888,7 +2888,7 @@
         <v>8</v>
       </c>
       <c r="F5" s="11">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G5" s="11">
         <v>10</v>
@@ -2897,7 +2897,7 @@
         <v>0</v>
       </c>
       <c r="I5" s="11">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J5" s="12">
         <f t="shared" si="0"/>

</xml_diff>

<commit_message>
Atualiza dados da homologacao - 24/07/2026 18:04
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E04B6AE-C57A-45A7-AB30-180A9E4FDBB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EBC30E3-1E7D-4056-B60F-D1B70FB802B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cenários homologação" sheetId="6" r:id="rId1"/>
@@ -1660,10 +1660,10 @@
     </row>
     <row r="16" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>82</v>
@@ -1725,7 +1725,7 @@
         <v>215</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>221</v>
+        <v>200</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>88</v>
@@ -2882,22 +2882,22 @@
         <v>1</v>
       </c>
       <c r="D5" s="11">
+        <v>2</v>
+      </c>
+      <c r="E5" s="11">
+        <v>5</v>
+      </c>
+      <c r="F5" s="11">
+        <v>15</v>
+      </c>
+      <c r="G5" s="11">
+        <v>11</v>
+      </c>
+      <c r="H5" s="11">
         <v>1</v>
       </c>
-      <c r="E5" s="11">
-        <v>8</v>
-      </c>
-      <c r="F5" s="11">
-        <v>16</v>
-      </c>
-      <c r="G5" s="11">
-        <v>10</v>
-      </c>
-      <c r="H5" s="11">
-        <v>0</v>
-      </c>
       <c r="I5" s="11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J5" s="12">
         <f t="shared" si="0"/>

</xml_diff>

<commit_message>
Atualiza dados da homologacao - 27/07/2026 15:04
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EBC30E3-1E7D-4056-B60F-D1B70FB802B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F42BA179-2E3A-4243-ABB9-005C5C72283C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cenários homologação" sheetId="6" r:id="rId1"/>
@@ -841,7 +841,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -867,6 +867,11 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1663,7 +1668,7 @@
         <v>215</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>216</v>
+        <v>201</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>82</v>
@@ -2372,7 +2377,7 @@
     <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39" s="4"/>
       <c r="B39" s="4" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="C39" s="4" t="s">
         <v>168</v>
@@ -2727,7 +2732,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E94EB92-949A-4861-8A92-72A5C32EFB43}">
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="21.77734375" customWidth="1"/>
@@ -2867,7 +2872,7 @@
         <v>5</v>
       </c>
       <c r="J4" s="12">
-        <f t="shared" ref="J4:J5" si="0">C4+D4+E4+F4+G4+H4+I4</f>
+        <f t="shared" ref="J4:J25" si="0">C4+D4+E4+F4+G4+H4+I4</f>
         <v>38</v>
       </c>
     </row>
@@ -2900,6 +2905,39 @@
         <v>3</v>
       </c>
       <c r="J5" s="12">
+        <f t="shared" si="0"/>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" s="9">
+        <v>0.625</v>
+      </c>
+      <c r="B6" s="13">
+        <v>46230</v>
+      </c>
+      <c r="C6" s="14">
+        <v>1</v>
+      </c>
+      <c r="D6" s="14">
+        <v>4</v>
+      </c>
+      <c r="E6" s="14">
+        <v>3</v>
+      </c>
+      <c r="F6" s="14">
+        <v>15</v>
+      </c>
+      <c r="G6" s="14">
+        <v>11</v>
+      </c>
+      <c r="H6" s="14">
+        <v>1</v>
+      </c>
+      <c r="I6" s="14">
+        <v>3</v>
+      </c>
+      <c r="J6" s="15">
         <f t="shared" si="0"/>
         <v>38</v>
       </c>

</xml_diff>

<commit_message>
Atualiza dados da homologacao - 28/07/2026 16:55
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F42BA179-2E3A-4243-ABB9-005C5C72283C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2713629C-73B7-4B24-AA52-E3EF3AB33C15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1668,7 +1668,7 @@
         <v>215</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>201</v>
+        <v>221</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>82</v>
@@ -1761,7 +1761,7 @@
         <v>215</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>201</v>
+        <v>216</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>91</v>
@@ -1947,7 +1947,7 @@
         <v>215</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>201</v>
+        <v>221</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>116</v>
@@ -2732,7 +2732,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E94EB92-949A-4861-8A92-72A5C32EFB43}">
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="21.77734375" customWidth="1"/>
@@ -2872,7 +2872,7 @@
         <v>5</v>
       </c>
       <c r="J4" s="12">
-        <f t="shared" ref="J4:J25" si="0">C4+D4+E4+F4+G4+H4+I4</f>
+        <f t="shared" ref="J4:J7" si="0">C4+D4+E4+F4+G4+H4+I4</f>
         <v>38</v>
       </c>
     </row>
@@ -2916,28 +2916,61 @@
       <c r="B6" s="13">
         <v>46230</v>
       </c>
-      <c r="C6" s="14">
+      <c r="C6" s="11">
         <v>1</v>
       </c>
-      <c r="D6" s="14">
+      <c r="D6" s="11">
         <v>4</v>
       </c>
-      <c r="E6" s="14">
+      <c r="E6" s="11">
         <v>3</v>
       </c>
-      <c r="F6" s="14">
+      <c r="F6" s="11">
         <v>15</v>
       </c>
-      <c r="G6" s="14">
+      <c r="G6" s="11">
         <v>11</v>
       </c>
-      <c r="H6" s="14">
+      <c r="H6" s="11">
         <v>1</v>
       </c>
-      <c r="I6" s="14">
+      <c r="I6" s="11">
         <v>3</v>
       </c>
-      <c r="J6" s="15">
+      <c r="J6" s="12">
+        <f t="shared" si="0"/>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7" s="9">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="B7" s="13">
+        <v>46231</v>
+      </c>
+      <c r="C7" s="14">
+        <v>1</v>
+      </c>
+      <c r="D7" s="14">
+        <v>5</v>
+      </c>
+      <c r="E7" s="14">
+        <v>4</v>
+      </c>
+      <c r="F7" s="14">
+        <v>15</v>
+      </c>
+      <c r="G7" s="14">
+        <v>11</v>
+      </c>
+      <c r="H7" s="14">
+        <v>2</v>
+      </c>
+      <c r="I7" s="14">
+        <v>0</v>
+      </c>
+      <c r="J7" s="15">
         <f t="shared" si="0"/>
         <v>38</v>
       </c>

</xml_diff>

<commit_message>
Atualiza dados da homologacao - 29/07/2026 16:21
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2713629C-73B7-4B24-AA52-E3EF3AB33C15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76796118-042A-477D-B35E-94B43DA10D74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -814,7 +814,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -837,11 +837,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -868,10 +879,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1186,6 +1199,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C39B64EC-B305-411B-89CD-90AE48303B1A}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:K44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1229,7 +1243,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>215</v>
       </c>
@@ -1260,7 +1274,7 @@
       <c r="J2" s="6"/>
       <c r="K2" s="6"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>215</v>
       </c>
@@ -1291,7 +1305,7 @@
       <c r="J3" s="6"/>
       <c r="K3" s="6"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>215</v>
       </c>
@@ -1322,7 +1336,7 @@
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
     </row>
-    <row r="5" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>215</v>
       </c>
@@ -1353,7 +1367,7 @@
       <c r="J5" s="6"/>
       <c r="K5" s="6"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>215</v>
       </c>
@@ -1384,7 +1398,7 @@
       <c r="J6" s="6"/>
       <c r="K6" s="6"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>210</v>
       </c>
@@ -1446,7 +1460,7 @@
       <c r="J8" s="6"/>
       <c r="K8" s="6"/>
     </row>
-    <row r="9" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>208</v>
       </c>
@@ -1477,7 +1491,7 @@
       <c r="J9" s="6"/>
       <c r="K9" s="6"/>
     </row>
-    <row r="10" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>211</v>
       </c>
@@ -1508,7 +1522,7 @@
       <c r="J10" s="6"/>
       <c r="K10" s="6"/>
     </row>
-    <row r="11" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>208</v>
       </c>
@@ -1539,7 +1553,7 @@
       <c r="J11" s="6"/>
       <c r="K11" s="6"/>
     </row>
-    <row r="12" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="86.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>208</v>
       </c>
@@ -1570,7 +1584,7 @@
       <c r="J12" s="6"/>
       <c r="K12" s="6"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>215</v>
       </c>
@@ -1601,7 +1615,7 @@
       <c r="J13" s="6"/>
       <c r="K13" s="6"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>210</v>
       </c>
@@ -1632,7 +1646,7 @@
       <c r="J14" s="6"/>
       <c r="K14" s="6"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>211</v>
       </c>
@@ -1694,7 +1708,7 @@
       <c r="J16" s="6"/>
       <c r="K16" s="6"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>215</v>
       </c>
@@ -1725,7 +1739,7 @@
       <c r="J17" s="6"/>
       <c r="K17" s="6"/>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>215</v>
       </c>
@@ -1756,7 +1770,7 @@
       <c r="J18" s="6"/>
       <c r="K18" s="6"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
         <v>215</v>
       </c>
@@ -1787,7 +1801,7 @@
       <c r="J19" s="6"/>
       <c r="K19" s="6"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>215</v>
       </c>
@@ -1818,7 +1832,7 @@
       <c r="J20" s="6"/>
       <c r="K20" s="6"/>
     </row>
-    <row r="21" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>215</v>
       </c>
@@ -1849,7 +1863,7 @@
       <c r="J21" s="6"/>
       <c r="K21" s="6"/>
     </row>
-    <row r="22" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>215</v>
       </c>
@@ -1880,7 +1894,7 @@
       <c r="J22" s="6"/>
       <c r="K22" s="6"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
         <v>215</v>
       </c>
@@ -1911,7 +1925,7 @@
       <c r="J23" s="6"/>
       <c r="K23" s="6"/>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
         <v>215</v>
       </c>
@@ -1973,7 +1987,7 @@
       <c r="J25" s="6"/>
       <c r="K25" s="6"/>
     </row>
-    <row r="26" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
         <v>215</v>
       </c>
@@ -2004,7 +2018,7 @@
       <c r="J26" s="6"/>
       <c r="K26" s="6"/>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
         <v>215</v>
       </c>
@@ -2035,7 +2049,7 @@
       <c r="J27" s="6"/>
       <c r="K27" s="6"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>215</v>
       </c>
@@ -2095,7 +2109,7 @@
       <c r="J29" s="6"/>
       <c r="K29" s="6"/>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
         <v>213</v>
       </c>
@@ -2126,7 +2140,7 @@
       <c r="J30" s="6"/>
       <c r="K30" s="6"/>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>215</v>
       </c>
@@ -2157,7 +2171,7 @@
       <c r="J31" s="6"/>
       <c r="K31" s="6"/>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
         <v>210</v>
       </c>
@@ -2188,7 +2202,7 @@
       <c r="J32" s="6"/>
       <c r="K32" s="6"/>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
         <v>210</v>
       </c>
@@ -2219,7 +2233,7 @@
       <c r="J33" s="6"/>
       <c r="K33" s="6"/>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
         <v>210</v>
       </c>
@@ -2250,7 +2264,7 @@
       <c r="J34" s="6"/>
       <c r="K34" s="6"/>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
         <v>215</v>
       </c>
@@ -2281,7 +2295,7 @@
       <c r="J35" s="6"/>
       <c r="K35" s="6"/>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
         <v>215</v>
       </c>
@@ -2312,7 +2326,7 @@
       <c r="J36" s="6"/>
       <c r="K36" s="6"/>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
         <v>215</v>
       </c>
@@ -2343,7 +2357,7 @@
       <c r="J37" s="6"/>
       <c r="K37" s="6"/>
     </row>
-    <row r="38" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:11" ht="86.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
         <v>215</v>
       </c>
@@ -2374,7 +2388,7 @@
       <c r="J38" s="6"/>
       <c r="K38" s="6"/>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" s="4"/>
       <c r="B39" s="4" t="s">
         <v>216</v>
@@ -2403,10 +2417,10 @@
       <c r="J39" s="6"/>
       <c r="K39" s="6"/>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" s="4"/>
       <c r="B40" s="4" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="C40" s="4" t="s">
         <v>173</v>
@@ -2432,10 +2446,10 @@
       <c r="J40" s="6"/>
       <c r="K40" s="6"/>
     </row>
-    <row r="41" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:11" ht="86.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" s="4"/>
       <c r="B41" s="4" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="C41" s="4" t="s">
         <v>176</v>
@@ -2521,7 +2535,7 @@
       <c r="J43" s="6"/>
       <c r="K43" s="6"/>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
         <v>208</v>
       </c>
@@ -2553,7 +2567,14 @@
       <c r="K44" s="6"/>
     </row>
   </sheetData>
-  <autoFilter ref="B1:B44" xr:uid="{C39B64EC-B305-411B-89CD-90AE48303B1A}"/>
+  <autoFilter ref="B1:B44" xr:uid="{C39B64EC-B305-411B-89CD-90AE48303B1A}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="Aguadando cenários"/>
+        <filter val="Em Correção"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -2732,7 +2753,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E94EB92-949A-4861-8A92-72A5C32EFB43}">
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="21.77734375" customWidth="1"/>
@@ -2872,7 +2893,7 @@
         <v>5</v>
       </c>
       <c r="J4" s="12">
-        <f t="shared" ref="J4:J7" si="0">C4+D4+E4+F4+G4+H4+I4</f>
+        <f t="shared" ref="J4:J8" si="0">C4+D4+E4+F4+G4+H4+I4</f>
         <v>38</v>
       </c>
     </row>
@@ -2949,28 +2970,61 @@
       <c r="B7" s="13">
         <v>46231</v>
       </c>
-      <c r="C7" s="14">
+      <c r="C7" s="11">
         <v>1</v>
       </c>
-      <c r="D7" s="14">
+      <c r="D7" s="11">
         <v>5</v>
       </c>
-      <c r="E7" s="14">
+      <c r="E7" s="11">
         <v>4</v>
       </c>
-      <c r="F7" s="14">
+      <c r="F7" s="11">
         <v>15</v>
       </c>
-      <c r="G7" s="14">
+      <c r="G7" s="11">
         <v>11</v>
       </c>
-      <c r="H7" s="14">
+      <c r="H7" s="11">
         <v>2</v>
       </c>
-      <c r="I7" s="14">
+      <c r="I7" s="11">
         <v>0</v>
       </c>
-      <c r="J7" s="15">
+      <c r="J7" s="12">
+        <f t="shared" si="0"/>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8" s="14">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="B8" s="15">
+        <v>46232</v>
+      </c>
+      <c r="C8" s="16">
+        <v>1</v>
+      </c>
+      <c r="D8" s="16">
+        <v>4</v>
+      </c>
+      <c r="E8" s="16">
+        <v>3</v>
+      </c>
+      <c r="F8" s="16">
+        <v>15</v>
+      </c>
+      <c r="G8" s="16">
+        <v>11</v>
+      </c>
+      <c r="H8" s="16">
+        <v>4</v>
+      </c>
+      <c r="I8" s="16">
+        <v>0</v>
+      </c>
+      <c r="J8" s="17">
         <f t="shared" si="0"/>
         <v>38</v>
       </c>

</xml_diff>

<commit_message>
Atualiza dados da homologacao - 30/07/2026  9:01
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76796118-042A-477D-B35E-94B43DA10D74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8502E56-F8AE-49AE-8936-19E2F7C59DCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cenários homologação" sheetId="6" r:id="rId1"/>
@@ -881,10 +881,10 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3007,10 +3007,10 @@
         <v>1</v>
       </c>
       <c r="D8" s="16">
+        <v>3</v>
+      </c>
+      <c r="E8" s="16">
         <v>4</v>
-      </c>
-      <c r="E8" s="16">
-        <v>3</v>
       </c>
       <c r="F8" s="16">
         <v>15</v>

</xml_diff>

<commit_message>
Atualiza dados da homologacao - 30/07/2026 16:53
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8502E56-F8AE-49AE-8936-19E2F7C59DCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E24C341-803A-4E95-A82C-9C894BF7D0CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cenários homologação" sheetId="6" r:id="rId1"/>
@@ -852,7 +852,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -885,6 +885,10 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1434,7 +1438,7 @@
         <v>211</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>221</v>
+        <v>207</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>43</v>
@@ -1682,7 +1686,7 @@
         <v>215</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>221</v>
+        <v>207</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>82</v>
@@ -1770,7 +1774,7 @@
       <c r="J18" s="6"/>
       <c r="K18" s="6"/>
     </row>
-    <row r="19" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
         <v>215</v>
       </c>
@@ -2388,7 +2392,7 @@
       <c r="J38" s="6"/>
       <c r="K38" s="6"/>
     </row>
-    <row r="39" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39" s="4"/>
       <c r="B39" s="4" t="s">
         <v>216</v>
@@ -2417,7 +2421,7 @@
       <c r="J39" s="6"/>
       <c r="K39" s="6"/>
     </row>
-    <row r="40" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" s="4"/>
       <c r="B40" s="4" t="s">
         <v>216</v>
@@ -2446,7 +2450,7 @@
       <c r="J40" s="6"/>
       <c r="K40" s="6"/>
     </row>
-    <row r="41" spans="1:11" ht="86.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A41" s="4"/>
       <c r="B41" s="4" t="s">
         <v>216</v>
@@ -2571,6 +2575,7 @@
     <filterColumn colId="0">
       <filters>
         <filter val="Aguadando cenários"/>
+        <filter val="Disponivel para Reteste"/>
         <filter val="Em Correção"/>
       </filters>
     </filterColumn>
@@ -2753,7 +2758,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E94EB92-949A-4861-8A92-72A5C32EFB43}">
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="21.77734375" customWidth="1"/>
@@ -2893,7 +2898,7 @@
         <v>5</v>
       </c>
       <c r="J4" s="12">
-        <f t="shared" ref="J4:J8" si="0">C4+D4+E4+F4+G4+H4+I4</f>
+        <f t="shared" ref="J4:J9" si="0">C4+D4+E4+F4+G4+H4+I4</f>
         <v>38</v>
       </c>
     </row>
@@ -3025,6 +3030,39 @@
         <v>0</v>
       </c>
       <c r="J8" s="17">
+        <f t="shared" si="0"/>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A9" s="14">
+        <v>0.70138888888888884</v>
+      </c>
+      <c r="B9" s="15">
+        <v>46233</v>
+      </c>
+      <c r="C9" s="18">
+        <v>1</v>
+      </c>
+      <c r="D9" s="18">
+        <v>2</v>
+      </c>
+      <c r="E9" s="18">
+        <v>3</v>
+      </c>
+      <c r="F9" s="18">
+        <v>15</v>
+      </c>
+      <c r="G9" s="18">
+        <v>13</v>
+      </c>
+      <c r="H9" s="18">
+        <v>4</v>
+      </c>
+      <c r="I9" s="18">
+        <v>0</v>
+      </c>
+      <c r="J9" s="19">
         <f t="shared" si="0"/>
         <v>38</v>
       </c>

</xml_diff>

<commit_message>
Atualiza dados da homologacao - 04/08/2026 14:37
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E24C341-803A-4E95-A82C-9C894BF7D0CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6D5A065-7831-4FA6-8BBF-1E79AD54E1CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cenários homologação" sheetId="6" r:id="rId1"/>
@@ -1203,7 +1203,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C39B64EC-B305-411B-89CD-90AE48303B1A}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:K44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1247,7 +1246,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>215</v>
       </c>
@@ -1278,7 +1277,7 @@
       <c r="J2" s="6"/>
       <c r="K2" s="6"/>
     </row>
-    <row r="3" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>215</v>
       </c>
@@ -1309,7 +1308,7 @@
       <c r="J3" s="6"/>
       <c r="K3" s="6"/>
     </row>
-    <row r="4" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>215</v>
       </c>
@@ -1340,7 +1339,7 @@
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
     </row>
-    <row r="5" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>215</v>
       </c>
@@ -1371,7 +1370,7 @@
       <c r="J5" s="6"/>
       <c r="K5" s="6"/>
     </row>
-    <row r="6" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>215</v>
       </c>
@@ -1402,7 +1401,7 @@
       <c r="J6" s="6"/>
       <c r="K6" s="6"/>
     </row>
-    <row r="7" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>210</v>
       </c>
@@ -1464,7 +1463,7 @@
       <c r="J8" s="6"/>
       <c r="K8" s="6"/>
     </row>
-    <row r="9" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>208</v>
       </c>
@@ -1495,7 +1494,7 @@
       <c r="J9" s="6"/>
       <c r="K9" s="6"/>
     </row>
-    <row r="10" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>211</v>
       </c>
@@ -1526,7 +1525,7 @@
       <c r="J10" s="6"/>
       <c r="K10" s="6"/>
     </row>
-    <row r="11" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>208</v>
       </c>
@@ -1557,7 +1556,7 @@
       <c r="J11" s="6"/>
       <c r="K11" s="6"/>
     </row>
-    <row r="12" spans="1:11" ht="86.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>208</v>
       </c>
@@ -1588,7 +1587,7 @@
       <c r="J12" s="6"/>
       <c r="K12" s="6"/>
     </row>
-    <row r="13" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>215</v>
       </c>
@@ -1619,7 +1618,7 @@
       <c r="J13" s="6"/>
       <c r="K13" s="6"/>
     </row>
-    <row r="14" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>210</v>
       </c>
@@ -1650,7 +1649,7 @@
       <c r="J14" s="6"/>
       <c r="K14" s="6"/>
     </row>
-    <row r="15" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>211</v>
       </c>
@@ -1712,7 +1711,7 @@
       <c r="J16" s="6"/>
       <c r="K16" s="6"/>
     </row>
-    <row r="17" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>215</v>
       </c>
@@ -1743,12 +1742,12 @@
       <c r="J17" s="6"/>
       <c r="K17" s="6"/>
     </row>
-    <row r="18" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>215</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>200</v>
+        <v>221</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>88</v>
@@ -1779,7 +1778,7 @@
         <v>215</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>216</v>
+        <v>207</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>91</v>
@@ -1805,7 +1804,7 @@
       <c r="J19" s="6"/>
       <c r="K19" s="6"/>
     </row>
-    <row r="20" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>215</v>
       </c>
@@ -1836,7 +1835,7 @@
       <c r="J20" s="6"/>
       <c r="K20" s="6"/>
     </row>
-    <row r="21" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>215</v>
       </c>
@@ -1867,7 +1866,7 @@
       <c r="J21" s="6"/>
       <c r="K21" s="6"/>
     </row>
-    <row r="22" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>215</v>
       </c>
@@ -1898,7 +1897,7 @@
       <c r="J22" s="6"/>
       <c r="K22" s="6"/>
     </row>
-    <row r="23" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
         <v>215</v>
       </c>
@@ -1929,7 +1928,7 @@
       <c r="J23" s="6"/>
       <c r="K23" s="6"/>
     </row>
-    <row r="24" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
         <v>215</v>
       </c>
@@ -1965,7 +1964,7 @@
         <v>215</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>116</v>
@@ -1991,7 +1990,7 @@
       <c r="J25" s="6"/>
       <c r="K25" s="6"/>
     </row>
-    <row r="26" spans="1:11" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
         <v>215</v>
       </c>
@@ -2022,7 +2021,7 @@
       <c r="J26" s="6"/>
       <c r="K26" s="6"/>
     </row>
-    <row r="27" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
         <v>215</v>
       </c>
@@ -2053,7 +2052,7 @@
       <c r="J27" s="6"/>
       <c r="K27" s="6"/>
     </row>
-    <row r="28" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>215</v>
       </c>
@@ -2113,7 +2112,7 @@
       <c r="J29" s="6"/>
       <c r="K29" s="6"/>
     </row>
-    <row r="30" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
         <v>213</v>
       </c>
@@ -2144,7 +2143,7 @@
       <c r="J30" s="6"/>
       <c r="K30" s="6"/>
     </row>
-    <row r="31" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>215</v>
       </c>
@@ -2175,7 +2174,7 @@
       <c r="J31" s="6"/>
       <c r="K31" s="6"/>
     </row>
-    <row r="32" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
         <v>210</v>
       </c>
@@ -2206,7 +2205,7 @@
       <c r="J32" s="6"/>
       <c r="K32" s="6"/>
     </row>
-    <row r="33" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
         <v>210</v>
       </c>
@@ -2237,7 +2236,7 @@
       <c r="J33" s="6"/>
       <c r="K33" s="6"/>
     </row>
-    <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
         <v>210</v>
       </c>
@@ -2268,7 +2267,7 @@
       <c r="J34" s="6"/>
       <c r="K34" s="6"/>
     </row>
-    <row r="35" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
         <v>215</v>
       </c>
@@ -2299,7 +2298,7 @@
       <c r="J35" s="6"/>
       <c r="K35" s="6"/>
     </row>
-    <row r="36" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
         <v>215</v>
       </c>
@@ -2330,7 +2329,7 @@
       <c r="J36" s="6"/>
       <c r="K36" s="6"/>
     </row>
-    <row r="37" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
         <v>215</v>
       </c>
@@ -2361,7 +2360,7 @@
       <c r="J37" s="6"/>
       <c r="K37" s="6"/>
     </row>
-    <row r="38" spans="1:11" ht="86.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
         <v>215</v>
       </c>
@@ -2453,7 +2452,7 @@
     <row r="41" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A41" s="4"/>
       <c r="B41" s="4" t="s">
-        <v>216</v>
+        <v>201</v>
       </c>
       <c r="C41" s="4" t="s">
         <v>176</v>
@@ -2482,7 +2481,7 @@
     <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A42" s="4"/>
       <c r="B42" s="4" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="C42" s="4" t="s">
         <v>179</v>
@@ -2513,7 +2512,7 @@
         <v>215</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>221</v>
+        <v>201</v>
       </c>
       <c r="C43" s="4" t="s">
         <v>185</v>
@@ -2539,7 +2538,7 @@
       <c r="J43" s="6"/>
       <c r="K43" s="6"/>
     </row>
-    <row r="44" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
         <v>208</v>
       </c>
@@ -2571,15 +2570,7 @@
       <c r="K44" s="6"/>
     </row>
   </sheetData>
-  <autoFilter ref="B1:B44" xr:uid="{C39B64EC-B305-411B-89CD-90AE48303B1A}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="Aguadando cenários"/>
-        <filter val="Disponivel para Reteste"/>
-        <filter val="Em Correção"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="B1:B44" xr:uid="{C39B64EC-B305-411B-89CD-90AE48303B1A}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -2758,7 +2749,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E94EB92-949A-4861-8A92-72A5C32EFB43}">
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="21.77734375" customWidth="1"/>
@@ -2898,7 +2889,7 @@
         <v>5</v>
       </c>
       <c r="J4" s="12">
-        <f t="shared" ref="J4:J9" si="0">C4+D4+E4+F4+G4+H4+I4</f>
+        <f t="shared" ref="J4:J10" si="0">C4+D4+E4+F4+G4+H4+I4</f>
         <v>38</v>
       </c>
     </row>
@@ -3041,28 +3032,61 @@
       <c r="B9" s="15">
         <v>46233</v>
       </c>
-      <c r="C9" s="18">
+      <c r="C9" s="16">
         <v>1</v>
       </c>
-      <c r="D9" s="18">
+      <c r="D9" s="16">
         <v>2</v>
       </c>
-      <c r="E9" s="18">
+      <c r="E9" s="16">
         <v>3</v>
       </c>
-      <c r="F9" s="18">
+      <c r="F9" s="16">
         <v>15</v>
       </c>
-      <c r="G9" s="18">
+      <c r="G9" s="16">
         <v>13</v>
       </c>
-      <c r="H9" s="18">
+      <c r="H9" s="16">
         <v>4</v>
       </c>
-      <c r="I9" s="18">
+      <c r="I9" s="16">
         <v>0</v>
       </c>
-      <c r="J9" s="19">
+      <c r="J9" s="17">
+        <f t="shared" si="0"/>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A10" s="14">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="B10" s="15">
+        <v>46238</v>
+      </c>
+      <c r="C10" s="18">
+        <v>1</v>
+      </c>
+      <c r="D10" s="18">
+        <v>2</v>
+      </c>
+      <c r="E10" s="18">
+        <v>0</v>
+      </c>
+      <c r="F10" s="18">
+        <v>15</v>
+      </c>
+      <c r="G10" s="18">
+        <v>14</v>
+      </c>
+      <c r="H10" s="18">
+        <v>4</v>
+      </c>
+      <c r="I10" s="18">
+        <v>2</v>
+      </c>
+      <c r="J10" s="19">
         <f t="shared" si="0"/>
         <v>38</v>
       </c>

</xml_diff>

<commit_message>
Atualiza dados da homologacao - 04/08/2026 17:27
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6D5A065-7831-4FA6-8BBF-1E79AD54E1CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83B966E0-13B2-48B2-9253-412B8CDDC417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cenários homologação" sheetId="6" r:id="rId1"/>
@@ -852,7 +852,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -885,10 +885,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1203,6 +1199,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C39B64EC-B305-411B-89CD-90AE48303B1A}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:K44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1246,7 +1243,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>215</v>
       </c>
@@ -1277,7 +1274,7 @@
       <c r="J2" s="6"/>
       <c r="K2" s="6"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>215</v>
       </c>
@@ -1308,7 +1305,7 @@
       <c r="J3" s="6"/>
       <c r="K3" s="6"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>215</v>
       </c>
@@ -1339,7 +1336,7 @@
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
     </row>
-    <row r="5" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>215</v>
       </c>
@@ -1370,7 +1367,7 @@
       <c r="J5" s="6"/>
       <c r="K5" s="6"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>215</v>
       </c>
@@ -1401,7 +1398,7 @@
       <c r="J6" s="6"/>
       <c r="K6" s="6"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>210</v>
       </c>
@@ -1432,7 +1429,7 @@
       <c r="J7" s="6"/>
       <c r="K7" s="6"/>
     </row>
-    <row r="8" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>211</v>
       </c>
@@ -1463,7 +1460,7 @@
       <c r="J8" s="6"/>
       <c r="K8" s="6"/>
     </row>
-    <row r="9" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>208</v>
       </c>
@@ -1494,7 +1491,7 @@
       <c r="J9" s="6"/>
       <c r="K9" s="6"/>
     </row>
-    <row r="10" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>211</v>
       </c>
@@ -1525,7 +1522,7 @@
       <c r="J10" s="6"/>
       <c r="K10" s="6"/>
     </row>
-    <row r="11" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>208</v>
       </c>
@@ -1556,7 +1553,7 @@
       <c r="J11" s="6"/>
       <c r="K11" s="6"/>
     </row>
-    <row r="12" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="86.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>208</v>
       </c>
@@ -1587,7 +1584,7 @@
       <c r="J12" s="6"/>
       <c r="K12" s="6"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>215</v>
       </c>
@@ -1618,7 +1615,7 @@
       <c r="J13" s="6"/>
       <c r="K13" s="6"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>210</v>
       </c>
@@ -1649,7 +1646,7 @@
       <c r="J14" s="6"/>
       <c r="K14" s="6"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>211</v>
       </c>
@@ -1680,7 +1677,7 @@
       <c r="J15" s="6"/>
       <c r="K15" s="6"/>
     </row>
-    <row r="16" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>215</v>
       </c>
@@ -1711,7 +1708,7 @@
       <c r="J16" s="6"/>
       <c r="K16" s="6"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>215</v>
       </c>
@@ -1773,7 +1770,7 @@
       <c r="J18" s="6"/>
       <c r="K18" s="6"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
         <v>215</v>
       </c>
@@ -1804,7 +1801,7 @@
       <c r="J19" s="6"/>
       <c r="K19" s="6"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>215</v>
       </c>
@@ -1835,7 +1832,7 @@
       <c r="J20" s="6"/>
       <c r="K20" s="6"/>
     </row>
-    <row r="21" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>215</v>
       </c>
@@ -1866,7 +1863,7 @@
       <c r="J21" s="6"/>
       <c r="K21" s="6"/>
     </row>
-    <row r="22" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>215</v>
       </c>
@@ -1897,7 +1894,7 @@
       <c r="J22" s="6"/>
       <c r="K22" s="6"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
         <v>215</v>
       </c>
@@ -1928,7 +1925,7 @@
       <c r="J23" s="6"/>
       <c r="K23" s="6"/>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
         <v>215</v>
       </c>
@@ -1964,7 +1961,7 @@
         <v>215</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>216</v>
+        <v>207</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>116</v>
@@ -1990,7 +1987,7 @@
       <c r="J25" s="6"/>
       <c r="K25" s="6"/>
     </row>
-    <row r="26" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
         <v>215</v>
       </c>
@@ -2021,7 +2018,7 @@
       <c r="J26" s="6"/>
       <c r="K26" s="6"/>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
         <v>215</v>
       </c>
@@ -2052,7 +2049,7 @@
       <c r="J27" s="6"/>
       <c r="K27" s="6"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>215</v>
       </c>
@@ -2112,7 +2109,7 @@
       <c r="J29" s="6"/>
       <c r="K29" s="6"/>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
         <v>213</v>
       </c>
@@ -2143,7 +2140,7 @@
       <c r="J30" s="6"/>
       <c r="K30" s="6"/>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>215</v>
       </c>
@@ -2174,7 +2171,7 @@
       <c r="J31" s="6"/>
       <c r="K31" s="6"/>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
         <v>210</v>
       </c>
@@ -2205,7 +2202,7 @@
       <c r="J32" s="6"/>
       <c r="K32" s="6"/>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
         <v>210</v>
       </c>
@@ -2236,7 +2233,7 @@
       <c r="J33" s="6"/>
       <c r="K33" s="6"/>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
         <v>210</v>
       </c>
@@ -2267,7 +2264,7 @@
       <c r="J34" s="6"/>
       <c r="K34" s="6"/>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
         <v>215</v>
       </c>
@@ -2298,7 +2295,7 @@
       <c r="J35" s="6"/>
       <c r="K35" s="6"/>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
         <v>215</v>
       </c>
@@ -2329,7 +2326,7 @@
       <c r="J36" s="6"/>
       <c r="K36" s="6"/>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
         <v>215</v>
       </c>
@@ -2360,7 +2357,7 @@
       <c r="J37" s="6"/>
       <c r="K37" s="6"/>
     </row>
-    <row r="38" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:11" ht="86.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
         <v>215</v>
       </c>
@@ -2391,10 +2388,10 @@
       <c r="J38" s="6"/>
       <c r="K38" s="6"/>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" s="4"/>
       <c r="B39" s="4" t="s">
-        <v>216</v>
+        <v>200</v>
       </c>
       <c r="C39" s="4" t="s">
         <v>168</v>
@@ -2423,7 +2420,7 @@
     <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" s="4"/>
       <c r="B40" s="4" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="C40" s="4" t="s">
         <v>173</v>
@@ -2452,7 +2449,7 @@
     <row r="41" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A41" s="4"/>
       <c r="B41" s="4" t="s">
-        <v>201</v>
+        <v>216</v>
       </c>
       <c r="C41" s="4" t="s">
         <v>176</v>
@@ -2512,7 +2509,7 @@
         <v>215</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>201</v>
+        <v>216</v>
       </c>
       <c r="C43" s="4" t="s">
         <v>185</v>
@@ -2538,7 +2535,7 @@
       <c r="J43" s="6"/>
       <c r="K43" s="6"/>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
         <v>208</v>
       </c>
@@ -2570,7 +2567,15 @@
       <c r="K44" s="6"/>
     </row>
   </sheetData>
-  <autoFilter ref="B1:B44" xr:uid="{C39B64EC-B305-411B-89CD-90AE48303B1A}"/>
+  <autoFilter ref="B1:B44" xr:uid="{C39B64EC-B305-411B-89CD-90AE48303B1A}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="Aguadando cenários"/>
+        <filter val="Disponivel para Reteste"/>
+        <filter val="Em Correção"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -3060,33 +3065,33 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="14">
-        <v>0.60416666666666663</v>
+        <v>0.70138888888888884</v>
       </c>
       <c r="B10" s="15">
         <v>46238</v>
       </c>
-      <c r="C10" s="18">
+      <c r="C10" s="16">
         <v>1</v>
       </c>
-      <c r="D10" s="18">
-        <v>2</v>
-      </c>
-      <c r="E10" s="18">
+      <c r="D10" s="16">
+        <v>1</v>
+      </c>
+      <c r="E10" s="16">
+        <v>1</v>
+      </c>
+      <c r="F10" s="16">
+        <v>17</v>
+      </c>
+      <c r="G10" s="16">
+        <v>15</v>
+      </c>
+      <c r="H10" s="16">
+        <v>3</v>
+      </c>
+      <c r="I10" s="16">
         <v>0</v>
       </c>
-      <c r="F10" s="18">
-        <v>15</v>
-      </c>
-      <c r="G10" s="18">
-        <v>14</v>
-      </c>
-      <c r="H10" s="18">
-        <v>4</v>
-      </c>
-      <c r="I10" s="18">
-        <v>2</v>
-      </c>
-      <c r="J10" s="19">
+      <c r="J10" s="17">
         <f t="shared" si="0"/>
         <v>38</v>
       </c>

</xml_diff>

<commit_message>
Atualiza dados da homologacao - 04/08/2026 17:38
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83B966E0-13B2-48B2-9253-412B8CDDC417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8004BEF-67C0-4695-A700-45604925EDB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8880" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cenários homologação" sheetId="6" r:id="rId1"/>
@@ -2420,7 +2420,7 @@
     <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" s="4"/>
       <c r="B40" s="4" t="s">
-        <v>221</v>
+        <v>200</v>
       </c>
       <c r="C40" s="4" t="s">
         <v>173</v>
@@ -3080,7 +3080,7 @@
         <v>1</v>
       </c>
       <c r="F10" s="16">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G10" s="16">
         <v>15</v>
@@ -3093,7 +3093,7 @@
       </c>
       <c r="J10" s="17">
         <f t="shared" si="0"/>
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza dados da homologacao - 04/08/2026 18:02
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8004BEF-67C0-4695-A700-45604925EDB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B82F8FCD-45E2-436E-82FB-A35293DF1F20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8880" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cenários homologação" sheetId="6" r:id="rId1"/>
@@ -2478,7 +2478,7 @@
     <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A42" s="4"/>
       <c r="B42" s="4" t="s">
-        <v>216</v>
+        <v>200</v>
       </c>
       <c r="C42" s="4" t="s">
         <v>179</v>
@@ -2509,7 +2509,7 @@
         <v>215</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>216</v>
+        <v>200</v>
       </c>
       <c r="C43" s="4" t="s">
         <v>185</v>

</xml_diff>

<commit_message>
Adiciona paginas SIBE com visao atual e evolucao, habilita card SIBE no portal
</commit_message>
<xml_diff>
--- a/CAF.xlsx
+++ b/CAF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B82F8FCD-45E2-436E-82FB-A35293DF1F20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B065E95B-B42D-47B1-8936-EA05848DE641}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1199,7 +1199,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C39B64EC-B305-411B-89CD-90AE48303B1A}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:K44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1243,7 +1242,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>215</v>
       </c>
@@ -1274,7 +1273,7 @@
       <c r="J2" s="6"/>
       <c r="K2" s="6"/>
     </row>
-    <row r="3" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>215</v>
       </c>
@@ -1305,7 +1304,7 @@
       <c r="J3" s="6"/>
       <c r="K3" s="6"/>
     </row>
-    <row r="4" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>215</v>
       </c>
@@ -1336,7 +1335,7 @@
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
     </row>
-    <row r="5" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>215</v>
       </c>
@@ -1367,7 +1366,7 @@
       <c r="J5" s="6"/>
       <c r="K5" s="6"/>
     </row>
-    <row r="6" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>215</v>
       </c>
@@ -1398,7 +1397,7 @@
       <c r="J6" s="6"/>
       <c r="K6" s="6"/>
     </row>
-    <row r="7" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>210</v>
       </c>
@@ -1429,7 +1428,7 @@
       <c r="J7" s="6"/>
       <c r="K7" s="6"/>
     </row>
-    <row r="8" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>211</v>
       </c>
@@ -1460,7 +1459,7 @@
       <c r="J8" s="6"/>
       <c r="K8" s="6"/>
     </row>
-    <row r="9" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>208</v>
       </c>
@@ -1491,7 +1490,7 @@
       <c r="J9" s="6"/>
       <c r="K9" s="6"/>
     </row>
-    <row r="10" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>211</v>
       </c>
@@ -1522,7 +1521,7 @@
       <c r="J10" s="6"/>
       <c r="K10" s="6"/>
     </row>
-    <row r="11" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>208</v>
       </c>
@@ -1553,7 +1552,7 @@
       <c r="J11" s="6"/>
       <c r="K11" s="6"/>
     </row>
-    <row r="12" spans="1:11" ht="86.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>208</v>
       </c>
@@ -1584,7 +1583,7 @@
       <c r="J12" s="6"/>
       <c r="K12" s="6"/>
     </row>
-    <row r="13" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>215</v>
       </c>
@@ -1615,7 +1614,7 @@
       <c r="J13" s="6"/>
       <c r="K13" s="6"/>
     </row>
-    <row r="14" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>210</v>
       </c>
@@ -1646,7 +1645,7 @@
       <c r="J14" s="6"/>
       <c r="K14" s="6"/>
     </row>
-    <row r="15" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>211</v>
       </c>
@@ -1677,7 +1676,7 @@
       <c r="J15" s="6"/>
       <c r="K15" s="6"/>
     </row>
-    <row r="16" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>215</v>
       </c>
@@ -1708,7 +1707,7 @@
       <c r="J16" s="6"/>
       <c r="K16" s="6"/>
     </row>
-    <row r="17" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>215</v>
       </c>
@@ -1770,7 +1769,7 @@
       <c r="J18" s="6"/>
       <c r="K18" s="6"/>
     </row>
-    <row r="19" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
         <v>215</v>
       </c>
@@ -1801,7 +1800,7 @@
       <c r="J19" s="6"/>
       <c r="K19" s="6"/>
     </row>
-    <row r="20" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>215</v>
       </c>
@@ -1832,7 +1831,7 @@
       <c r="J20" s="6"/>
       <c r="K20" s="6"/>
     </row>
-    <row r="21" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>215</v>
       </c>
@@ -1863,7 +1862,7 @@
       <c r="J21" s="6"/>
       <c r="K21" s="6"/>
     </row>
-    <row r="22" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>215</v>
       </c>
@@ -1894,7 +1893,7 @@
       <c r="J22" s="6"/>
       <c r="K22" s="6"/>
     </row>
-    <row r="23" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
         <v>215</v>
       </c>
@@ -1925,7 +1924,7 @@
       <c r="J23" s="6"/>
       <c r="K23" s="6"/>
     </row>
-    <row r="24" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
         <v>215</v>
       </c>
@@ -1987,7 +1986,7 @@
       <c r="J25" s="6"/>
       <c r="K25" s="6"/>
     </row>
-    <row r="26" spans="1:11" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
         <v>215</v>
       </c>
@@ -2018,7 +2017,7 @@
       <c r="J26" s="6"/>
       <c r="K26" s="6"/>
     </row>
-    <row r="27" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
         <v>215</v>
       </c>
@@ -2049,7 +2048,7 @@
       <c r="J27" s="6"/>
       <c r="K27" s="6"/>
     </row>
-    <row r="28" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>215</v>
       </c>
@@ -2109,7 +2108,7 @@
       <c r="J29" s="6"/>
       <c r="K29" s="6"/>
     </row>
-    <row r="30" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
         <v>213</v>
       </c>
@@ -2140,7 +2139,7 @@
       <c r="J30" s="6"/>
       <c r="K30" s="6"/>
     </row>
-    <row r="31" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>215</v>
       </c>
@@ -2171,7 +2170,7 @@
       <c r="J31" s="6"/>
       <c r="K31" s="6"/>
     </row>
-    <row r="32" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
         <v>210</v>
       </c>
@@ -2202,7 +2201,7 @@
       <c r="J32" s="6"/>
       <c r="K32" s="6"/>
     </row>
-    <row r="33" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
         <v>210</v>
       </c>
@@ -2233,7 +2232,7 @@
       <c r="J33" s="6"/>
       <c r="K33" s="6"/>
     </row>
-    <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
         <v>210</v>
       </c>
@@ -2264,7 +2263,7 @@
       <c r="J34" s="6"/>
       <c r="K34" s="6"/>
     </row>
-    <row r="35" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
         <v>215</v>
       </c>
@@ -2295,7 +2294,7 @@
       <c r="J35" s="6"/>
       <c r="K35" s="6"/>
     </row>
-    <row r="36" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
         <v>215</v>
       </c>
@@ -2326,7 +2325,7 @@
       <c r="J36" s="6"/>
       <c r="K36" s="6"/>
     </row>
-    <row r="37" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
         <v>215</v>
       </c>
@@ -2357,7 +2356,7 @@
       <c r="J37" s="6"/>
       <c r="K37" s="6"/>
     </row>
-    <row r="38" spans="1:11" ht="86.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
         <v>215</v>
       </c>
@@ -2388,7 +2387,7 @@
       <c r="J38" s="6"/>
       <c r="K38" s="6"/>
     </row>
-    <row r="39" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39" s="4"/>
       <c r="B39" s="4" t="s">
         <v>200</v>
@@ -2535,7 +2534,7 @@
       <c r="J43" s="6"/>
       <c r="K43" s="6"/>
     </row>
-    <row r="44" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
         <v>208</v>
       </c>
@@ -2567,15 +2566,7 @@
       <c r="K44" s="6"/>
     </row>
   </sheetData>
-  <autoFilter ref="B1:B44" xr:uid="{C39B64EC-B305-411B-89CD-90AE48303B1A}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="Aguadando cenários"/>
-        <filter val="Disponivel para Reteste"/>
-        <filter val="Em Correção"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="B1:B44" xr:uid="{C39B64EC-B305-411B-89CD-90AE48303B1A}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">

</xml_diff>